<commit_message>
Fusion study: passive static-charge channel plus alarm rules
fusion_study.py adds charge sharing at contact (sourced body and fabric
capacitances, walking charge and decay, humidity, ADC noise) to the active
sweep and compares three alarm rules for coverage by body location and
unwanted prompts per hour, as a function of the still-unmeasured body
voltage between two people. Logs 16 new values from 9 papers in the
workbook. Model and demo unchanged.
</commit_message>
<xml_diff>
--- a/docs/SparshaGuard_paper_values.xlsx
+++ b/docs/SparshaGuard_paper_values.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference List" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Values from Papers'!$A$1:$J$136</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Values from Papers'!$A$1:$J$161</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J136"/>
+  <dimension ref="A1:J161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5016,70 +5016,68 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="inlineStr">
+      <c r="A102" s="5" t="n">
+        <v>89</v>
+      </c>
+      <c r="B102" s="5" t="inlineStr">
+        <is>
+          <t>Body-to-body capacitance at 1 m (analytic)</t>
+        </is>
+      </c>
+      <c r="C102" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="D102" s="5" t="inlineStr">
+        <is>
+          <t>pF</t>
+        </is>
+      </c>
+      <c r="E102" s="5" t="inlineStr">
+        <is>
+          <t>Two 1.8 m people</t>
+        </is>
+      </c>
+      <c r="F102" s="5" t="inlineStr">
+        <is>
+          <t>Nath et al. 2021</t>
+        </is>
+      </c>
+      <c r="G102" s="5" t="inlineStr">
+        <is>
+          <t>M. Nath et al. (S. Sen group, Purdue) (2021). "Inter-Body Coupling in Electro-Quasistatic Human Body Communication: Theory and Analysis of Security and Interference Properties". Scientific Reports.</t>
+        </is>
+      </c>
+      <c r="H102" s="5" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="I102" s="6" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2003.13329</t>
+        </is>
+      </c>
+      <c r="J102" s="5" t="inlineStr">
+        <is>
+          <t>Fusion study (doc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
         <is>
           <t>Agarwal &amp; Sahu 2010  —  Indian Journal of Plastic Surgery 43(1)</t>
         </is>
       </c>
-      <c r="B102" s="3" t="n"/>
-      <c r="C102" s="3" t="n"/>
-      <c r="D102" s="3" t="n"/>
-      <c r="E102" s="3" t="n"/>
-      <c r="F102" s="3" t="n"/>
-      <c r="G102" s="3" t="n"/>
-      <c r="H102" s="3" t="n"/>
-      <c r="I102" s="3" t="n"/>
-      <c r="J102" s="4" t="n"/>
-    </row>
-    <row r="103">
-      <c r="A103" s="5" t="n">
-        <v>89</v>
-      </c>
-      <c r="B103" s="5" t="inlineStr">
-        <is>
-          <t>Hand area (palmar, incl. fingers), men</t>
-        </is>
-      </c>
-      <c r="C103" s="5" t="inlineStr">
-        <is>
-          <t>146.5 ± 15.1</t>
-        </is>
-      </c>
-      <c r="D103" s="5" t="inlineStr">
-        <is>
-          <t>cm²</t>
-        </is>
-      </c>
-      <c r="E103" s="5" t="inlineStr">
-        <is>
-          <t>Indian adults 18–60, n = 150; Supports 40–80 cm² grab contact</t>
-        </is>
-      </c>
-      <c r="F103" s="5" t="inlineStr">
-        <is>
-          <t>Agarwal &amp; Sahu 2010</t>
-        </is>
-      </c>
-      <c r="G103" s="5" t="inlineStr">
-        <is>
-          <t>P. Agarwal, S. Sahu (2010). "Determination of hand and palm area as a ratio of body surface area in Indian population". Indian Journal of Plastic Surgery 43(1).</t>
-        </is>
-      </c>
-      <c r="H103" s="5" t="inlineStr">
-        <is>
-          <t>Results</t>
-        </is>
-      </c>
-      <c r="I103" s="6" t="inlineStr">
-        <is>
-          <t>https://www.thieme-connect.de/products/ejournals/pdf/10.1055/s-0039-1699403.pdf</t>
-        </is>
-      </c>
-      <c r="J103" s="5" t="inlineStr">
-        <is>
-          <t>Yes (in model)</t>
-        </is>
-      </c>
+      <c r="B103" s="3" t="n"/>
+      <c r="C103" s="3" t="n"/>
+      <c r="D103" s="3" t="n"/>
+      <c r="E103" s="3" t="n"/>
+      <c r="F103" s="3" t="n"/>
+      <c r="G103" s="3" t="n"/>
+      <c r="H103" s="3" t="n"/>
+      <c r="I103" s="3" t="n"/>
+      <c r="J103" s="4" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="5" t="n">
@@ -5087,12 +5085,12 @@
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>Hand area (palmar, incl. fingers), women</t>
+          <t>Hand area (palmar, incl. fingers), men</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>132.4 ± 14.1</t>
+          <t>146.5 ± 15.1</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
@@ -5102,7 +5100,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t>n = 150</t>
+          <t>Indian adults 18–60, n = 150; Supports 40–80 cm² grab contact</t>
         </is>
       </c>
       <c r="F104" s="5" t="inlineStr">
@@ -5137,12 +5135,12 @@
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>Palm area, men</t>
+          <t>Hand area (palmar, incl. fingers), women</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>77.9 ± 10.3</t>
+          <t>132.4 ± 14.1</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
@@ -5150,7 +5148,11 @@
           <t>cm²</t>
         </is>
       </c>
-      <c r="E105" s="5" t="inlineStr"/>
+      <c r="E105" s="5" t="inlineStr">
+        <is>
+          <t>n = 150</t>
+        </is>
+      </c>
       <c r="F105" s="5" t="inlineStr">
         <is>
           <t>Agarwal &amp; Sahu 2010</t>
@@ -5173,7 +5175,7 @@
       </c>
       <c r="J105" s="5" t="inlineStr">
         <is>
-          <t>Background only</t>
+          <t>Yes (in model)</t>
         </is>
       </c>
     </row>
@@ -5183,12 +5185,12 @@
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>Palm area, women</t>
+          <t>Palm area, men</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>73.7 ± 9.1</t>
+          <t>77.9 ± 10.3</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
@@ -5229,111 +5231,111 @@
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
+          <t>Palm area, women</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>73.7 ± 9.1</t>
+        </is>
+      </c>
+      <c r="D107" s="5" t="inlineStr">
+        <is>
+          <t>cm²</t>
+        </is>
+      </c>
+      <c r="E107" s="5" t="inlineStr"/>
+      <c r="F107" s="5" t="inlineStr">
+        <is>
+          <t>Agarwal &amp; Sahu 2010</t>
+        </is>
+      </c>
+      <c r="G107" s="5" t="inlineStr">
+        <is>
+          <t>P. Agarwal, S. Sahu (2010). "Determination of hand and palm area as a ratio of body surface area in Indian population". Indian Journal of Plastic Surgery 43(1).</t>
+        </is>
+      </c>
+      <c r="H107" s="5" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I107" s="6" t="inlineStr">
+        <is>
+          <t>https://www.thieme-connect.de/products/ejournals/pdf/10.1055/s-0039-1699403.pdf</t>
+        </is>
+      </c>
+      <c r="J107" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="5" t="n">
+        <v>94</v>
+      </c>
+      <c r="B108" s="5" t="inlineStr">
+        <is>
           <t>Hand as % of body surface area</t>
         </is>
       </c>
-      <c r="C107" s="5" t="inlineStr">
+      <c r="C108" s="5" t="inlineStr">
         <is>
           <t>0.92</t>
         </is>
       </c>
-      <c r="D107" s="5" t="inlineStr">
+      <c r="D108" s="5" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E107" s="5" t="inlineStr">
+      <c r="E108" s="5" t="inlineStr">
         <is>
           <t>Men and women</t>
         </is>
       </c>
-      <c r="F107" s="5" t="inlineStr">
+      <c r="F108" s="5" t="inlineStr">
         <is>
           <t>Agarwal &amp; Sahu 2010</t>
         </is>
       </c>
-      <c r="G107" s="5" t="inlineStr">
+      <c r="G108" s="5" t="inlineStr">
         <is>
           <t>P. Agarwal, S. Sahu (2010). "Determination of hand and palm area as a ratio of body surface area in Indian population". Indian Journal of Plastic Surgery 43(1).</t>
         </is>
       </c>
-      <c r="H107" s="5" t="inlineStr">
+      <c r="H108" s="5" t="inlineStr">
         <is>
           <t>Results</t>
         </is>
       </c>
-      <c r="I107" s="6" t="inlineStr">
+      <c r="I108" s="6" t="inlineStr">
         <is>
           <t>https://www.thieme-connect.de/products/ejournals/pdf/10.1055/s-0039-1699403.pdf</t>
         </is>
       </c>
-      <c r="J107" s="5" t="inlineStr">
+      <c r="J108" s="5" t="inlineStr">
         <is>
           <t>Background only</t>
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" s="2" t="inlineStr">
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
         <is>
           <t>TI SNOA926 2015  —  Application report</t>
         </is>
       </c>
-      <c r="B108" s="3" t="n"/>
-      <c r="C108" s="3" t="n"/>
-      <c r="D108" s="3" t="n"/>
-      <c r="E108" s="3" t="n"/>
-      <c r="F108" s="3" t="n"/>
-      <c r="G108" s="3" t="n"/>
-      <c r="H108" s="3" t="n"/>
-      <c r="I108" s="3" t="n"/>
-      <c r="J108" s="4" t="n"/>
-    </row>
-    <row r="109">
-      <c r="A109" s="5" t="n">
-        <v>94</v>
-      </c>
-      <c r="B109" s="5" t="inlineStr">
-        <is>
-          <t>Unshielded ground parasitic</t>
-        </is>
-      </c>
-      <c r="C109" s="5" t="inlineStr">
-        <is>
-          <t>&gt; 100 (can be)</t>
-        </is>
-      </c>
-      <c r="D109" s="5" t="inlineStr">
-        <is>
-          <t>pF</t>
-        </is>
-      </c>
-      <c r="E109" s="5" t="inlineStr"/>
-      <c r="F109" s="5" t="inlineStr">
-        <is>
-          <t>TI SNOA926 2015</t>
-        </is>
-      </c>
-      <c r="G109" s="5" t="inlineStr">
-        <is>
-          <t>Texas Instruments (2015). "Capacitive Sensing: Ins and Outs of Active Shielding (SNOA926A)". Application report.</t>
-        </is>
-      </c>
-      <c r="H109" s="5" t="inlineStr">
-        <is>
-          <t>Fig. 4</t>
-        </is>
-      </c>
-      <c r="I109" s="6" t="inlineStr">
-        <is>
-          <t>https://www.ti.com/lit/pdf/SNOA926</t>
-        </is>
-      </c>
-      <c r="J109" s="5" t="inlineStr">
-        <is>
-          <t>Background only</t>
-        </is>
-      </c>
+      <c r="B109" s="3" t="n"/>
+      <c r="C109" s="3" t="n"/>
+      <c r="D109" s="3" t="n"/>
+      <c r="E109" s="3" t="n"/>
+      <c r="F109" s="3" t="n"/>
+      <c r="G109" s="3" t="n"/>
+      <c r="H109" s="3" t="n"/>
+      <c r="I109" s="3" t="n"/>
+      <c r="J109" s="4" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="5" t="n">
@@ -5341,24 +5343,20 @@
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>Rejection of object behind sensor (3.6 cm)</t>
+          <t>Unshielded ground parasitic</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>50.9 / 61.1 / 76.3</t>
+          <t>&gt; 100 (can be)</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>% reduction</t>
-        </is>
-      </c>
-      <c r="E110" s="5" t="inlineStr">
-        <is>
-          <t>Same-size shield / 200% shield / ring + shield; Residual 24–49%</t>
-        </is>
-      </c>
+          <t>pF</t>
+        </is>
+      </c>
+      <c r="E110" s="5" t="inlineStr"/>
       <c r="F110" s="5" t="inlineStr">
         <is>
           <t>TI SNOA926 2015</t>
@@ -5371,7 +5369,7 @@
       </c>
       <c r="H110" s="5" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Fig. 4</t>
         </is>
       </c>
       <c r="I110" s="6" t="inlineStr">
@@ -5381,7 +5379,7 @@
       </c>
       <c r="J110" s="5" t="inlineStr">
         <is>
-          <t>Yes (in model)</t>
+          <t>Background only</t>
         </is>
       </c>
     </row>
@@ -5391,12 +5389,12 @@
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>Rejection of object at side (1 cm)</t>
+          <t>Rejection of object behind sensor (3.6 cm)</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>37.2 / 70.6 / 77.0</t>
+          <t>50.9 / 61.1 / 76.3</t>
         </is>
       </c>
       <c r="D111" s="5" t="inlineStr">
@@ -5406,7 +5404,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t>Same three configurations; Residual 23–63%</t>
+          <t>Same-size shield / 200% shield / ring + shield; Residual 24–49%</t>
         </is>
       </c>
       <c r="F111" s="5" t="inlineStr">
@@ -5441,12 +5439,12 @@
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>Rejection of object at side (5 cm)</t>
+          <t>Rejection of object at side (1 cm)</t>
         </is>
       </c>
       <c r="C112" s="5" t="inlineStr">
         <is>
-          <t>34.2 / 64.6 / 75.0</t>
+          <t>37.2 / 70.6 / 77.0</t>
         </is>
       </c>
       <c r="D112" s="5" t="inlineStr">
@@ -5456,7 +5454,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t>Same three configurations</t>
+          <t>Same three configurations; Residual 23–63%</t>
         </is>
       </c>
       <c r="F112" s="5" t="inlineStr">
@@ -5481,7 +5479,7 @@
       </c>
       <c r="J112" s="5" t="inlineStr">
         <is>
-          <t>Background only</t>
+          <t>Yes (in model)</t>
         </is>
       </c>
     </row>
@@ -5491,115 +5489,115 @@
       </c>
       <c r="B113" s="5" t="inlineStr">
         <is>
+          <t>Rejection of object at side (5 cm)</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>34.2 / 64.6 / 75.0</t>
+        </is>
+      </c>
+      <c r="D113" s="5" t="inlineStr">
+        <is>
+          <t>% reduction</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>Same three configurations</t>
+        </is>
+      </c>
+      <c r="F113" s="5" t="inlineStr">
+        <is>
+          <t>TI SNOA926 2015</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr">
+        <is>
+          <t>Texas Instruments (2015). "Capacitive Sensing: Ins and Outs of Active Shielding (SNOA926A)". Application report.</t>
+        </is>
+      </c>
+      <c r="H113" s="5" t="inlineStr">
+        <is>
+          <t>Table 1</t>
+        </is>
+      </c>
+      <c r="I113" s="6" t="inlineStr">
+        <is>
+          <t>https://www.ti.com/lit/pdf/SNOA926</t>
+        </is>
+      </c>
+      <c r="J113" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="5" t="n">
+        <v>99</v>
+      </c>
+      <c r="B114" s="5" t="inlineStr">
+        <is>
           <t>Loss of wanted sensitivity (top, 1 cm)</t>
         </is>
       </c>
-      <c r="C113" s="5" t="inlineStr">
+      <c r="C114" s="5" t="inlineStr">
         <is>
           <t>23.6 / 26.5 / 39.3</t>
         </is>
       </c>
-      <c r="D113" s="5" t="inlineStr">
+      <c r="D114" s="5" t="inlineStr">
         <is>
           <t>% reduction</t>
         </is>
       </c>
-      <c r="E113" s="5" t="inlineStr">
+      <c r="E114" s="5" t="inlineStr">
         <is>
           <t>Same three configurations; Shield also costs some signal</t>
         </is>
       </c>
-      <c r="F113" s="5" t="inlineStr">
+      <c r="F114" s="5" t="inlineStr">
         <is>
           <t>TI SNOA926 2015</t>
         </is>
       </c>
-      <c r="G113" s="5" t="inlineStr">
+      <c r="G114" s="5" t="inlineStr">
         <is>
           <t>Texas Instruments (2015). "Capacitive Sensing: Ins and Outs of Active Shielding (SNOA926A)". Application report.</t>
         </is>
       </c>
-      <c r="H113" s="5" t="inlineStr">
+      <c r="H114" s="5" t="inlineStr">
         <is>
           <t>Table 1</t>
         </is>
       </c>
-      <c r="I113" s="6" t="inlineStr">
+      <c r="I114" s="6" t="inlineStr">
         <is>
           <t>https://www.ti.com/lit/pdf/SNOA926</t>
         </is>
       </c>
-      <c r="J113" s="5" t="inlineStr">
+      <c r="J114" s="5" t="inlineStr">
         <is>
           <t>Background only</t>
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="2" t="inlineStr">
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
         <is>
           <t>Hackaday ADC test  —  Hackaday.io</t>
         </is>
       </c>
-      <c r="B114" s="3" t="n"/>
-      <c r="C114" s="3" t="n"/>
-      <c r="D114" s="3" t="n"/>
-      <c r="E114" s="3" t="n"/>
-      <c r="F114" s="3" t="n"/>
-      <c r="G114" s="3" t="n"/>
-      <c r="H114" s="3" t="n"/>
-      <c r="I114" s="3" t="n"/>
-      <c r="J114" s="4" t="n"/>
-    </row>
-    <row r="115">
-      <c r="A115" s="5" t="n">
-        <v>99</v>
-      </c>
-      <c r="B115" s="5" t="inlineStr">
-        <is>
-          <t>ESP32 built-in ADC fluctuation</t>
-        </is>
-      </c>
-      <c r="C115" s="5" t="inlineStr">
-        <is>
-          <t>~21.8</t>
-        </is>
-      </c>
-      <c r="D115" s="5" t="inlineStr">
-        <is>
-          <t>mV</t>
-        </is>
-      </c>
-      <c r="E115" s="5" t="inlineStr">
-        <is>
-          <t>Unclear if std. dev. or p-p; ≈27 LSB at 3.3 V; Weak source</t>
-        </is>
-      </c>
-      <c r="F115" s="5" t="inlineStr">
-        <is>
-          <t>Hackaday ADC test</t>
-        </is>
-      </c>
-      <c r="G115" s="5" t="inlineStr">
-        <is>
-          <t>Hackaday.io project (n.d.). "ADC performance: Arduino vs ESP32 vs ADS1115". Hackaday.io.</t>
-        </is>
-      </c>
-      <c r="H115" s="5" t="inlineStr">
-        <is>
-          <t>Results</t>
-        </is>
-      </c>
-      <c r="I115" s="6" t="inlineStr">
-        <is>
-          <t>https://hackaday.io/project/205380-adc-performance-arduino-vs-esp32-vs-ads1115</t>
-        </is>
-      </c>
-      <c r="J115" s="5" t="inlineStr">
-        <is>
-          <t>Yes (in model)</t>
-        </is>
-      </c>
+      <c r="B115" s="3" t="n"/>
+      <c r="C115" s="3" t="n"/>
+      <c r="D115" s="3" t="n"/>
+      <c r="E115" s="3" t="n"/>
+      <c r="F115" s="3" t="n"/>
+      <c r="G115" s="3" t="n"/>
+      <c r="H115" s="3" t="n"/>
+      <c r="I115" s="3" t="n"/>
+      <c r="J115" s="4" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="5" t="n">
@@ -5607,12 +5605,12 @@
       </c>
       <c r="B116" s="5" t="inlineStr">
         <is>
-          <t>Arduino ADC fluctuation</t>
+          <t>ESP32 built-in ADC fluctuation</t>
         </is>
       </c>
       <c r="C116" s="5" t="inlineStr">
         <is>
-          <t>~4.2</t>
+          <t>~21.8</t>
         </is>
       </c>
       <c r="D116" s="5" t="inlineStr">
@@ -5620,7 +5618,11 @@
           <t>mV</t>
         </is>
       </c>
-      <c r="E116" s="5" t="inlineStr"/>
+      <c r="E116" s="5" t="inlineStr">
+        <is>
+          <t>Unclear if std. dev. or p-p; ≈27 LSB at 3.3 V; Weak source</t>
+        </is>
+      </c>
       <c r="F116" s="5" t="inlineStr">
         <is>
           <t>Hackaday ADC test</t>
@@ -5643,7 +5645,7 @@
       </c>
       <c r="J116" s="5" t="inlineStr">
         <is>
-          <t>Background only</t>
+          <t>Yes (in model)</t>
         </is>
       </c>
     </row>
@@ -5653,115 +5655,111 @@
       </c>
       <c r="B117" s="5" t="inlineStr">
         <is>
+          <t>Arduino ADC fluctuation</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>~4.2</t>
+        </is>
+      </c>
+      <c r="D117" s="5" t="inlineStr">
+        <is>
+          <t>mV</t>
+        </is>
+      </c>
+      <c r="E117" s="5" t="inlineStr"/>
+      <c r="F117" s="5" t="inlineStr">
+        <is>
+          <t>Hackaday ADC test</t>
+        </is>
+      </c>
+      <c r="G117" s="5" t="inlineStr">
+        <is>
+          <t>Hackaday.io project (n.d.). "ADC performance: Arduino vs ESP32 vs ADS1115". Hackaday.io.</t>
+        </is>
+      </c>
+      <c r="H117" s="5" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I117" s="6" t="inlineStr">
+        <is>
+          <t>https://hackaday.io/project/205380-adc-performance-arduino-vs-esp32-vs-ads1115</t>
+        </is>
+      </c>
+      <c r="J117" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="5" t="n">
+        <v>102</v>
+      </c>
+      <c r="B118" s="5" t="inlineStr">
+        <is>
           <t>ADS1115 fluctuation</t>
         </is>
       </c>
-      <c r="C117" s="5" t="inlineStr">
+      <c r="C118" s="5" t="inlineStr">
         <is>
           <t>~2</t>
         </is>
       </c>
-      <c r="D117" s="5" t="inlineStr">
+      <c r="D118" s="5" t="inlineStr">
         <is>
           <t>mV</t>
         </is>
       </c>
-      <c r="E117" s="5" t="inlineStr">
+      <c r="E118" s="5" t="inlineStr">
         <is>
           <t>External ADC option</t>
         </is>
       </c>
-      <c r="F117" s="5" t="inlineStr">
+      <c r="F118" s="5" t="inlineStr">
         <is>
           <t>Hackaday ADC test</t>
         </is>
       </c>
-      <c r="G117" s="5" t="inlineStr">
+      <c r="G118" s="5" t="inlineStr">
         <is>
           <t>Hackaday.io project (n.d.). "ADC performance: Arduino vs ESP32 vs ADS1115". Hackaday.io.</t>
         </is>
       </c>
-      <c r="H117" s="5" t="inlineStr">
+      <c r="H118" s="5" t="inlineStr">
         <is>
           <t>Results</t>
         </is>
       </c>
-      <c r="I117" s="6" t="inlineStr">
+      <c r="I118" s="6" t="inlineStr">
         <is>
           <t>https://hackaday.io/project/205380-adc-performance-arduino-vs-esp32-vs-ads1115</t>
         </is>
       </c>
-      <c r="J117" s="5" t="inlineStr">
+      <c r="J118" s="5" t="inlineStr">
         <is>
           <t>Background only</t>
         </is>
       </c>
     </row>
-    <row r="118">
-      <c r="A118" s="2" t="inlineStr">
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
         <is>
           <t>Espressif ADC blog 2025  —  developer.espressif.com</t>
         </is>
       </c>
-      <c r="B118" s="3" t="n"/>
-      <c r="C118" s="3" t="n"/>
-      <c r="D118" s="3" t="n"/>
-      <c r="E118" s="3" t="n"/>
-      <c r="F118" s="3" t="n"/>
-      <c r="G118" s="3" t="n"/>
-      <c r="H118" s="3" t="n"/>
-      <c r="I118" s="3" t="n"/>
-      <c r="J118" s="4" t="n"/>
-    </row>
-    <row r="119">
-      <c r="A119" s="5" t="n">
-        <v>102</v>
-      </c>
-      <c r="B119" s="5" t="inlineStr">
-        <is>
-          <t>ESP32 calibrated error</t>
-        </is>
-      </c>
-      <c r="C119" s="5" t="inlineStr">
-        <is>
-          <t>&lt; 30</t>
-        </is>
-      </c>
-      <c r="D119" s="5" t="inlineStr">
-        <is>
-          <t>mV</t>
-        </is>
-      </c>
-      <c r="E119" s="5" t="inlineStr">
-        <is>
-          <t>Accuracy, not noise</t>
-        </is>
-      </c>
-      <c r="F119" s="5" t="inlineStr">
-        <is>
-          <t>Espressif ADC blog 2025</t>
-        </is>
-      </c>
-      <c r="G119" s="5" t="inlineStr">
-        <is>
-          <t>Espressif Systems (2025). "ADC performance (developer blog)". developer.espressif.com.</t>
-        </is>
-      </c>
-      <c r="H119" s="5" t="inlineStr">
-        <is>
-          <t>Results</t>
-        </is>
-      </c>
-      <c r="I119" s="6" t="inlineStr">
-        <is>
-          <t>https://developer.espressif.com/blog/2025/08/adc-performance/</t>
-        </is>
-      </c>
-      <c r="J119" s="5" t="inlineStr">
-        <is>
-          <t>Background only</t>
-        </is>
-      </c>
+      <c r="B119" s="3" t="n"/>
+      <c r="C119" s="3" t="n"/>
+      <c r="D119" s="3" t="n"/>
+      <c r="E119" s="3" t="n"/>
+      <c r="F119" s="3" t="n"/>
+      <c r="G119" s="3" t="n"/>
+      <c r="H119" s="3" t="n"/>
+      <c r="I119" s="3" t="n"/>
+      <c r="J119" s="4" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="5" t="n">
@@ -5769,12 +5767,12 @@
       </c>
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>ESP32-S3 calibrated error</t>
+          <t>ESP32 calibrated error</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
         <is>
-          <t>−30 to 0</t>
+          <t>&lt; 30</t>
         </is>
       </c>
       <c r="D120" s="5" t="inlineStr">
@@ -5782,7 +5780,11 @@
           <t>mV</t>
         </is>
       </c>
-      <c r="E120" s="5" t="inlineStr"/>
+      <c r="E120" s="5" t="inlineStr">
+        <is>
+          <t>Accuracy, not noise</t>
+        </is>
+      </c>
       <c r="F120" s="5" t="inlineStr">
         <is>
           <t>Espressif ADC blog 2025</t>
@@ -5815,24 +5817,20 @@
       </c>
       <c r="B121" s="5" t="inlineStr">
         <is>
-          <t>ESP32 / ESP32-S3 DNL, INL</t>
+          <t>ESP32-S3 calibrated error</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>±7, ±12 / ±4, ±8</t>
+          <t>−30 to 0</t>
         </is>
       </c>
       <c r="D121" s="5" t="inlineStr">
         <is>
-          <t>LSB</t>
-        </is>
-      </c>
-      <c r="E121" s="5" t="inlineStr">
-        <is>
-          <t>Datasheet values</t>
-        </is>
-      </c>
+          <t>mV</t>
+        </is>
+      </c>
+      <c r="E121" s="5" t="inlineStr"/>
       <c r="F121" s="5" t="inlineStr">
         <is>
           <t>Espressif ADC blog 2025</t>
@@ -5845,7 +5843,7 @@
       </c>
       <c r="H121" s="5" t="inlineStr">
         <is>
-          <t>Table 1</t>
+          <t>Results</t>
         </is>
       </c>
       <c r="I121" s="6" t="inlineStr">
@@ -5865,20 +5863,24 @@
       </c>
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>ESP32 ADC sample rate</t>
+          <t>ESP32 / ESP32-S3 DNL, INL</t>
         </is>
       </c>
       <c r="C122" s="5" t="inlineStr">
         <is>
-          <t>200 k (RTC) / 2 M (DIG)</t>
+          <t>±7, ±12 / ±4, ±8</t>
         </is>
       </c>
       <c r="D122" s="5" t="inlineStr">
         <is>
-          <t>samples/s</t>
-        </is>
-      </c>
-      <c r="E122" s="5" t="inlineStr"/>
+          <t>LSB</t>
+        </is>
+      </c>
+      <c r="E122" s="5" t="inlineStr">
+        <is>
+          <t>Datasheet values</t>
+        </is>
+      </c>
       <c r="F122" s="5" t="inlineStr">
         <is>
           <t>Espressif ADC blog 2025</t>
@@ -5911,115 +5913,111 @@
       </c>
       <c r="B123" s="5" t="inlineStr">
         <is>
+          <t>ESP32 ADC sample rate</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>200 k (RTC) / 2 M (DIG)</t>
+        </is>
+      </c>
+      <c r="D123" s="5" t="inlineStr">
+        <is>
+          <t>samples/s</t>
+        </is>
+      </c>
+      <c r="E123" s="5" t="inlineStr"/>
+      <c r="F123" s="5" t="inlineStr">
+        <is>
+          <t>Espressif ADC blog 2025</t>
+        </is>
+      </c>
+      <c r="G123" s="5" t="inlineStr">
+        <is>
+          <t>Espressif Systems (2025). "ADC performance (developer blog)". developer.espressif.com.</t>
+        </is>
+      </c>
+      <c r="H123" s="5" t="inlineStr">
+        <is>
+          <t>Table 1</t>
+        </is>
+      </c>
+      <c r="I123" s="6" t="inlineStr">
+        <is>
+          <t>https://developer.espressif.com/blog/2025/08/adc-performance/</t>
+        </is>
+      </c>
+      <c r="J123" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="5" t="n">
+        <v>107</v>
+      </c>
+      <c r="B124" s="5" t="inlineStr">
+        <is>
           <t>Noise advice</t>
         </is>
       </c>
-      <c r="C123" s="5" t="inlineStr">
+      <c r="C124" s="5" t="inlineStr">
         <is>
           <t>100 nF on ADC input; multisampling</t>
         </is>
       </c>
-      <c r="D123" s="5" t="inlineStr">
+      <c r="D124" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E123" s="5" t="inlineStr">
+      <c r="E124" s="5" t="inlineStr">
         <is>
           <t>No figures given</t>
         </is>
       </c>
-      <c r="F123" s="5" t="inlineStr">
+      <c r="F124" s="5" t="inlineStr">
         <is>
           <t>Espressif ADC blog 2025</t>
         </is>
       </c>
-      <c r="G123" s="5" t="inlineStr">
+      <c r="G124" s="5" t="inlineStr">
         <is>
           <t>Espressif Systems (2025). "ADC performance (developer blog)". developer.espressif.com.</t>
         </is>
       </c>
-      <c r="H123" s="5" t="inlineStr">
+      <c r="H124" s="5" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="I123" s="6" t="inlineStr">
+      <c r="I124" s="6" t="inlineStr">
         <is>
           <t>https://developer.espressif.com/blog/2025/08/adc-performance/</t>
         </is>
       </c>
-      <c r="J123" s="5" t="inlineStr">
+      <c r="J124" s="5" t="inlineStr">
         <is>
           <t>Background only</t>
         </is>
       </c>
     </row>
-    <row r="124">
-      <c r="A124" s="2" t="inlineStr">
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
         <is>
           <t>Desco ESD table  —  descoindustries.com</t>
         </is>
       </c>
-      <c r="B124" s="3" t="n"/>
-      <c r="C124" s="3" t="n"/>
-      <c r="D124" s="3" t="n"/>
-      <c r="E124" s="3" t="n"/>
-      <c r="F124" s="3" t="n"/>
-      <c r="G124" s="3" t="n"/>
-      <c r="H124" s="3" t="n"/>
-      <c r="I124" s="3" t="n"/>
-      <c r="J124" s="4" t="n"/>
-    </row>
-    <row r="125">
-      <c r="A125" s="5" t="n">
-        <v>107</v>
-      </c>
-      <c r="B125" s="5" t="inlineStr">
-        <is>
-          <t>Body voltage, walking on vinyl floor</t>
-        </is>
-      </c>
-      <c r="C125" s="5" t="inlineStr">
-        <is>
-          <t>250 – 12,000</t>
-        </is>
-      </c>
-      <c r="D125" s="5" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="E125" s="5" t="inlineStr">
-        <is>
-          <t>65-90% / 10-20% relative humidity</t>
-        </is>
-      </c>
-      <c r="F125" s="5" t="inlineStr">
-        <is>
-          <t>Desco ESD table</t>
-        </is>
-      </c>
-      <c r="G125" s="5" t="inlineStr">
-        <is>
-          <t>Desco Industries (n.d.). "Typical Electrostatic Voltages". descoindustries.com.</t>
-        </is>
-      </c>
-      <c r="H125" s="5" t="inlineStr">
-        <is>
-          <t>Table</t>
-        </is>
-      </c>
-      <c r="I125" s="6" t="inlineStr">
-        <is>
-          <t>https://www.descoindustries.com/AboutESD/Voltage.aspx</t>
-        </is>
-      </c>
-      <c r="J125" s="5" t="inlineStr">
-        <is>
-          <t>Whole-body study (doc)</t>
-        </is>
-      </c>
+      <c r="B125" s="3" t="n"/>
+      <c r="C125" s="3" t="n"/>
+      <c r="D125" s="3" t="n"/>
+      <c r="E125" s="3" t="n"/>
+      <c r="F125" s="3" t="n"/>
+      <c r="G125" s="3" t="n"/>
+      <c r="H125" s="3" t="n"/>
+      <c r="I125" s="3" t="n"/>
+      <c r="J125" s="4" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="5" t="n">
@@ -6027,405 +6025,1350 @@
       </c>
       <c r="B126" s="5" t="inlineStr">
         <is>
+          <t>Body voltage, walking on vinyl floor</t>
+        </is>
+      </c>
+      <c r="C126" s="5" t="inlineStr">
+        <is>
+          <t>250 – 12,000</t>
+        </is>
+      </c>
+      <c r="D126" s="5" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="E126" s="5" t="inlineStr">
+        <is>
+          <t>65-90% / 10-20% relative humidity</t>
+        </is>
+      </c>
+      <c r="F126" s="5" t="inlineStr">
+        <is>
+          <t>Desco ESD table</t>
+        </is>
+      </c>
+      <c r="G126" s="5" t="inlineStr">
+        <is>
+          <t>Desco Industries (n.d.). "Typical Electrostatic Voltages". descoindustries.com.</t>
+        </is>
+      </c>
+      <c r="H126" s="5" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="I126" s="6" t="inlineStr">
+        <is>
+          <t>https://www.descoindustries.com/AboutESD/Voltage.aspx</t>
+        </is>
+      </c>
+      <c r="J126" s="5" t="inlineStr">
+        <is>
+          <t>Whole-body study (doc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="5" t="n">
+        <v>109</v>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
           <t>Body voltage, walking on carpet</t>
         </is>
       </c>
-      <c r="C126" s="5" t="inlineStr">
+      <c r="C127" s="5" t="inlineStr">
         <is>
           <t>1,500 – 35,000</t>
         </is>
       </c>
-      <c r="D126" s="5" t="inlineStr">
+      <c r="D127" s="5" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="E126" s="5" t="inlineStr">
+      <c r="E127" s="5" t="inlineStr">
         <is>
           <t>65-90% / 10-20% relative humidity</t>
         </is>
       </c>
-      <c r="F126" s="5" t="inlineStr">
+      <c r="F127" s="5" t="inlineStr">
         <is>
           <t>Desco ESD table</t>
         </is>
       </c>
-      <c r="G126" s="5" t="inlineStr">
+      <c r="G127" s="5" t="inlineStr">
         <is>
           <t>Desco Industries (n.d.). "Typical Electrostatic Voltages". descoindustries.com.</t>
         </is>
       </c>
-      <c r="H126" s="5" t="inlineStr">
+      <c r="H127" s="5" t="inlineStr">
         <is>
           <t>Table</t>
         </is>
       </c>
-      <c r="I126" s="6" t="inlineStr">
+      <c r="I127" s="6" t="inlineStr">
         <is>
           <t>https://www.descoindustries.com/AboutESD/Voltage.aspx</t>
         </is>
       </c>
-      <c r="J126" s="5" t="inlineStr">
+      <c r="J127" s="5" t="inlineStr">
         <is>
           <t>Whole-body study (doc)</t>
         </is>
       </c>
     </row>
-    <row r="127">
-      <c r="A127" s="2" t="inlineStr">
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
         <is>
           <t>Jonassen (walking)  —  In Compliance Magazine</t>
         </is>
       </c>
-      <c r="B127" s="3" t="n"/>
-      <c r="C127" s="3" t="n"/>
-      <c r="D127" s="3" t="n"/>
-      <c r="E127" s="3" t="n"/>
-      <c r="F127" s="3" t="n"/>
-      <c r="G127" s="3" t="n"/>
-      <c r="H127" s="3" t="n"/>
-      <c r="I127" s="3" t="n"/>
-      <c r="J127" s="4" t="n"/>
-    </row>
-    <row r="128">
-      <c r="A128" s="5" t="n">
-        <v>109</v>
-      </c>
-      <c r="B128" s="5" t="inlineStr">
+      <c r="B128" s="3" t="n"/>
+      <c r="C128" s="3" t="n"/>
+      <c r="D128" s="3" t="n"/>
+      <c r="E128" s="3" t="n"/>
+      <c r="F128" s="3" t="n"/>
+      <c r="G128" s="3" t="n"/>
+      <c r="H128" s="3" t="n"/>
+      <c r="I128" s="3" t="n"/>
+      <c r="J128" s="4" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="5" t="n">
+        <v>110</v>
+      </c>
+      <c r="B129" s="5" t="inlineStr">
         <is>
           <t>Body voltage from walking on vinyl (measured)</t>
         </is>
       </c>
-      <c r="C128" s="5" t="inlineStr">
+      <c r="C129" s="5" t="inlineStr">
         <is>
           <t>up to ~3,500</t>
         </is>
       </c>
-      <c r="D128" s="5" t="inlineStr">
+      <c r="D129" s="5" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="E128" s="5" t="inlineStr">
+      <c r="E129" s="5" t="inlineStr">
         <is>
           <t>Insulating floor</t>
         </is>
       </c>
-      <c r="F128" s="5" t="inlineStr">
+      <c r="F129" s="5" t="inlineStr">
         <is>
           <t>Jonassen (walking)</t>
         </is>
       </c>
-      <c r="G128" s="5" t="inlineStr">
+      <c r="G129" s="5" t="inlineStr">
         <is>
           <t>N. Jonassen (n.d.). "Charging by Walking (Mr. Static column)". In Compliance Magazine.</t>
         </is>
       </c>
-      <c r="H128" s="5" t="inlineStr">
+      <c r="H129" s="5" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="I128" s="6" t="inlineStr">
+      <c r="I129" s="6" t="inlineStr">
         <is>
           <t>https://incompliancemag.com/charging-by-walking/</t>
         </is>
       </c>
-      <c r="J128" s="5" t="inlineStr">
+      <c r="J129" s="5" t="inlineStr">
         <is>
           <t>Whole-body study (doc)</t>
         </is>
       </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="2" t="inlineStr">
-        <is>
-          <t>Bian et al. 2019  —  IEEE PerCom Workshops</t>
-        </is>
-      </c>
-      <c r="B129" s="3" t="n"/>
-      <c r="C129" s="3" t="n"/>
-      <c r="D129" s="3" t="n"/>
-      <c r="E129" s="3" t="n"/>
-      <c r="F129" s="3" t="n"/>
-      <c r="G129" s="3" t="n"/>
-      <c r="H129" s="3" t="n"/>
-      <c r="I129" s="3" t="n"/>
-      <c r="J129" s="4" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="5" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B130" s="5" t="inlineStr">
         <is>
+          <t>Peak walking voltage formula</t>
+        </is>
+      </c>
+      <c r="C130" s="5" t="inlineStr">
+        <is>
+          <t>V_max = R · n · Δq</t>
+        </is>
+      </c>
+      <c r="D130" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E130" s="5" t="inlineStr">
+        <is>
+          <t>R to ground, n steps per second, Δq charge per step</t>
+        </is>
+      </c>
+      <c r="F130" s="5" t="inlineStr">
+        <is>
+          <t>Jonassen (walking)</t>
+        </is>
+      </c>
+      <c r="G130" s="5" t="inlineStr">
+        <is>
+          <t>N. Jonassen (n.d.). "Charging by Walking (Mr. Static column)". In Compliance Magazine.</t>
+        </is>
+      </c>
+      <c r="H130" s="5" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="I130" s="6" t="inlineStr">
+        <is>
+          <t>https://incompliancemag.com/charging-by-walking/</t>
+        </is>
+      </c>
+      <c r="J130" s="5" t="inlineStr">
+        <is>
+          <t>Fusion study (doc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="5" t="n">
+        <v>112</v>
+      </c>
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>Body resistance to ground from initial decay</t>
+        </is>
+      </c>
+      <c r="C131" s="5" t="inlineStr">
+        <is>
+          <t>≈ 2 × 10^10</t>
+        </is>
+      </c>
+      <c r="D131" s="5" t="inlineStr">
+        <is>
+          <t>Ω</t>
+        </is>
+      </c>
+      <c r="E131" s="5" t="inlineStr">
+        <is>
+          <t>Walking test, decay after stopping</t>
+        </is>
+      </c>
+      <c r="F131" s="5" t="inlineStr">
+        <is>
+          <t>Jonassen (walking)</t>
+        </is>
+      </c>
+      <c r="G131" s="5" t="inlineStr">
+        <is>
+          <t>N. Jonassen (n.d.). "Charging by Walking (Mr. Static column)". In Compliance Magazine.</t>
+        </is>
+      </c>
+      <c r="H131" s="5" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="I131" s="6" t="inlineStr">
+        <is>
+          <t>https://incompliancemag.com/charging-by-walking/</t>
+        </is>
+      </c>
+      <c r="J131" s="5" t="inlineStr">
+        <is>
+          <t>Fusion study (doc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>Bian et al. 2019  —  IEEE PerCom Workshops</t>
+        </is>
+      </c>
+      <c r="B132" s="3" t="n"/>
+      <c r="C132" s="3" t="n"/>
+      <c r="D132" s="3" t="n"/>
+      <c r="E132" s="3" t="n"/>
+      <c r="F132" s="3" t="n"/>
+      <c r="G132" s="3" t="n"/>
+      <c r="H132" s="3" t="n"/>
+      <c r="I132" s="3" t="n"/>
+      <c r="J132" s="4" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="5" t="n">
+        <v>113</v>
+      </c>
+      <c r="B133" s="5" t="inlineStr">
+        <is>
           <t>Wrist passive field sensor sensitivity</t>
         </is>
       </c>
-      <c r="C130" s="5" t="inlineStr">
+      <c r="C133" s="5" t="inlineStr">
         <is>
           <t>microvolt-level</t>
         </is>
       </c>
-      <c r="D130" s="5" t="inlineStr">
+      <c r="D133" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E130" s="5" t="inlineStr">
+      <c r="E133" s="5" t="inlineStr">
         <is>
           <t>Wrist-worn, passive; Qualitative</t>
         </is>
       </c>
-      <c r="F130" s="5" t="inlineStr">
+      <c r="F133" s="5" t="inlineStr">
         <is>
           <t>Bian et al. 2019</t>
         </is>
       </c>
-      <c r="G130" s="5" t="inlineStr">
+      <c r="G133" s="5" t="inlineStr">
         <is>
           <t>S. Bian, V. F. Rey, J. Younas, P. Lukowicz (2019). "Wrist-Worn Capacitive Sensor for Activity and Physical Collaboration Recognition". IEEE PerCom Workshops.</t>
         </is>
       </c>
-      <c r="H130" s="5" t="inlineStr">
+      <c r="H133" s="5" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="I130" s="6" t="inlineStr">
+      <c r="I133" s="6" t="inlineStr">
         <is>
           <t>https://dfki.de/web/forschung/projekte-publikationen/publikation/10312</t>
         </is>
       </c>
-      <c r="J130" s="5" t="inlineStr">
+      <c r="J133" s="5" t="inlineStr">
         <is>
           <t>Whole-body study (doc)</t>
         </is>
       </c>
     </row>
-    <row r="131">
-      <c r="A131" s="2" t="inlineStr">
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
         <is>
           <t>Bian, Liu, Lukowicz 2025  —  arXiv:2507.13520</t>
         </is>
       </c>
-      <c r="B131" s="3" t="n"/>
-      <c r="C131" s="3" t="n"/>
-      <c r="D131" s="3" t="n"/>
-      <c r="E131" s="3" t="n"/>
-      <c r="F131" s="3" t="n"/>
-      <c r="G131" s="3" t="n"/>
-      <c r="H131" s="3" t="n"/>
-      <c r="I131" s="3" t="n"/>
-      <c r="J131" s="4" t="n"/>
-    </row>
-    <row r="132">
-      <c r="A132" s="5" t="n">
-        <v>111</v>
-      </c>
-      <c r="B132" s="5" t="inlineStr">
+      <c r="B134" s="3" t="n"/>
+      <c r="C134" s="3" t="n"/>
+      <c r="D134" s="3" t="n"/>
+      <c r="E134" s="3" t="n"/>
+      <c r="F134" s="3" t="n"/>
+      <c r="G134" s="3" t="n"/>
+      <c r="H134" s="3" t="n"/>
+      <c r="I134" s="3" t="n"/>
+      <c r="J134" s="4" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="5" t="n">
+        <v>114</v>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
         <is>
           <t>ProxiBand: approaching person detected (TPR)</t>
         </is>
       </c>
-      <c r="C132" s="5" t="inlineStr">
+      <c r="C135" s="5" t="inlineStr">
         <is>
           <t>74.3 / 46</t>
         </is>
       </c>
-      <c r="D132" s="5" t="inlineStr">
+      <c r="D135" s="5" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E132" s="5" t="inlineStr">
+      <c r="E135" s="5" t="inlineStr">
         <is>
           <t>Indoor / outdoor</t>
         </is>
       </c>
-      <c r="F132" s="5" t="inlineStr">
+      <c r="F135" s="5" t="inlineStr">
         <is>
           <t>Bian, Liu, Lukowicz 2025</t>
         </is>
       </c>
-      <c r="G132" s="5" t="inlineStr">
+      <c r="G135" s="5" t="inlineStr">
         <is>
           <t>S. Bian, M. Liu, P. Lukowicz (2025). "Passive Body-Area Electrostatic Field (Human Body Capacitance) for Ubiquitous Computing". arXiv:2507.13520.</t>
         </is>
       </c>
-      <c r="H132" s="5" t="inlineStr">
+      <c r="H135" s="5" t="inlineStr">
         <is>
           <t>Overview text</t>
         </is>
       </c>
-      <c r="I132" s="6" t="inlineStr">
+      <c r="I135" s="6" t="inlineStr">
         <is>
           <t>https://arxiv.org/html/2507.13520v1</t>
         </is>
       </c>
-      <c r="J132" s="5" t="inlineStr">
+      <c r="J135" s="5" t="inlineStr">
         <is>
           <t>Whole-body study (doc)</t>
         </is>
       </c>
     </row>
-    <row r="133">
-      <c r="A133" s="2" t="inlineStr">
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
         <is>
           <t>Kurita 2016  —  Electrostatics Joint Conference</t>
         </is>
       </c>
-      <c r="B133" s="3" t="n"/>
-      <c r="C133" s="3" t="n"/>
-      <c r="D133" s="3" t="n"/>
-      <c r="E133" s="3" t="n"/>
-      <c r="F133" s="3" t="n"/>
-      <c r="G133" s="3" t="n"/>
-      <c r="H133" s="3" t="n"/>
-      <c r="I133" s="3" t="n"/>
-      <c r="J133" s="4" t="n"/>
-    </row>
-    <row r="134">
-      <c r="A134" s="5" t="n">
-        <v>112</v>
-      </c>
-      <c r="B134" s="5" t="inlineStr">
+      <c r="B136" s="3" t="n"/>
+      <c r="C136" s="3" t="n"/>
+      <c r="D136" s="3" t="n"/>
+      <c r="E136" s="3" t="n"/>
+      <c r="F136" s="3" t="n"/>
+      <c r="G136" s="3" t="n"/>
+      <c r="H136" s="3" t="n"/>
+      <c r="I136" s="3" t="n"/>
+      <c r="J136" s="4" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="5" t="n">
+        <v>115</v>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
         <is>
           <t>Contact moment from electrostatic induction current</t>
         </is>
       </c>
-      <c r="C134" s="5" t="inlineStr">
+      <c r="C137" s="5" t="inlineStr">
         <is>
           <t>detected</t>
         </is>
       </c>
-      <c r="D134" s="5" t="inlineStr">
+      <c r="D137" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E134" s="5" t="inlineStr">
+      <c r="E137" s="5" t="inlineStr">
         <is>
           <t>Contact electrification; Qualitative</t>
         </is>
       </c>
-      <c r="F134" s="5" t="inlineStr">
+      <c r="F137" s="5" t="inlineStr">
         <is>
           <t>Kurita 2016</t>
         </is>
       </c>
-      <c r="G134" s="5" t="inlineStr">
+      <c r="G137" s="5" t="inlineStr">
         <is>
           <t>K. Kurita (2016). "Detection method for contact electrification based on electrostatic induction". Electrostatics Joint Conference.</t>
         </is>
       </c>
-      <c r="H134" s="5" t="inlineStr">
+      <c r="H137" s="5" t="inlineStr">
         <is>
           <t>Results</t>
         </is>
       </c>
-      <c r="I134" s="6" t="inlineStr">
+      <c r="I137" s="6" t="inlineStr">
         <is>
           <t>https://electrostatics.org/wp-content/uploads/2023/08/G12.pdf</t>
         </is>
       </c>
-      <c r="J134" s="5" t="inlineStr">
+      <c r="J137" s="5" t="inlineStr">
         <is>
           <t>Whole-body study (doc)</t>
         </is>
       </c>
     </row>
-    <row r="135">
-      <c r="A135" s="2" t="inlineStr">
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
         <is>
           <t>Elfekey et al. 2016  —  Sensors 16(12):2049</t>
         </is>
       </c>
-      <c r="B135" s="3" t="n"/>
-      <c r="C135" s="3" t="n"/>
-      <c r="D135" s="3" t="n"/>
-      <c r="E135" s="3" t="n"/>
-      <c r="F135" s="3" t="n"/>
-      <c r="G135" s="3" t="n"/>
-      <c r="H135" s="3" t="n"/>
-      <c r="I135" s="3" t="n"/>
-      <c r="J135" s="4" t="n"/>
-    </row>
-    <row r="136">
-      <c r="A136" s="5" t="n">
-        <v>113</v>
-      </c>
-      <c r="B136" s="5" t="inlineStr">
+      <c r="B138" s="3" t="n"/>
+      <c r="C138" s="3" t="n"/>
+      <c r="D138" s="3" t="n"/>
+      <c r="E138" s="3" t="n"/>
+      <c r="F138" s="3" t="n"/>
+      <c r="G138" s="3" t="n"/>
+      <c r="H138" s="3" t="n"/>
+      <c r="I138" s="3" t="n"/>
+      <c r="J138" s="4" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="5" t="n">
+        <v>116</v>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
         <is>
           <t>Touch sensing from induced 50 Hz field on body</t>
         </is>
       </c>
-      <c r="C136" s="5" t="inlineStr">
+      <c r="C139" s="5" t="inlineStr">
         <is>
           <t>demonstrated</t>
         </is>
       </c>
-      <c r="D136" s="5" t="inlineStr">
+      <c r="D139" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E136" s="5" t="inlineStr">
+      <c r="E139" s="5" t="inlineStr">
         <is>
           <t>Mains ELF field; Qualitative</t>
         </is>
       </c>
-      <c r="F136" s="5" t="inlineStr">
+      <c r="F139" s="5" t="inlineStr">
         <is>
           <t>Elfekey et al. 2016</t>
         </is>
       </c>
-      <c r="G136" s="5" t="inlineStr">
+      <c r="G139" s="5" t="inlineStr">
         <is>
           <t>H. Elfekey, H. A. Bastawrous, S. Okamoto (2016). "A Touch Sensing Technique Using the Effects of Extremely Low Frequency Fields on the Human Body". Sensors 16(12):2049.</t>
         </is>
       </c>
-      <c r="H136" s="5" t="inlineStr">
+      <c r="H139" s="5" t="inlineStr">
         <is>
           <t>Results</t>
         </is>
       </c>
-      <c r="I136" s="6" t="inlineStr">
+      <c r="I139" s="6" t="inlineStr">
         <is>
           <t>https://doi.org/10.3390/s16122049</t>
         </is>
       </c>
-      <c r="J136" s="5" t="inlineStr">
+      <c r="J139" s="5" t="inlineStr">
         <is>
           <t>Whole-body study (doc)</t>
         </is>
       </c>
     </row>
+    <row r="140">
+      <c r="A140" s="5" t="n">
+        <v>117</v>
+      </c>
+      <c r="B140" s="5" t="inlineStr">
+        <is>
+          <t>Hum at the controller input, touching vs not touching</t>
+        </is>
+      </c>
+      <c r="C140" s="5" t="inlineStr">
+        <is>
+          <t>&gt; 4 / &lt; 0.5</t>
+        </is>
+      </c>
+      <c r="D140" s="5" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="E140" s="5" t="inlineStr">
+        <is>
+          <t>Their sensing circuit, indoor mains field; Circuit-specific levels</t>
+        </is>
+      </c>
+      <c r="F140" s="5" t="inlineStr">
+        <is>
+          <t>Elfekey et al. 2016</t>
+        </is>
+      </c>
+      <c r="G140" s="5" t="inlineStr">
+        <is>
+          <t>H. Elfekey, H. A. Bastawrous, S. Okamoto (2016). "A Touch Sensing Technique Using the Effects of Extremely Low Frequency Fields on the Human Body". Sensors 16(12):2049.</t>
+        </is>
+      </c>
+      <c r="H140" s="5" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I140" s="6" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/s16122049</t>
+        </is>
+      </c>
+      <c r="J140" s="5" t="inlineStr">
+        <is>
+          <t>Fusion study (doc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>GKVK Bengaluru weather normals  —  uasbangalore.edu.in</t>
+        </is>
+      </c>
+      <c r="B141" s="3" t="n"/>
+      <c r="C141" s="3" t="n"/>
+      <c r="D141" s="3" t="n"/>
+      <c r="E141" s="3" t="n"/>
+      <c r="F141" s="3" t="n"/>
+      <c r="G141" s="3" t="n"/>
+      <c r="H141" s="3" t="n"/>
+      <c r="I141" s="3" t="n"/>
+      <c r="J141" s="4" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="5" t="n">
+        <v>118</v>
+      </c>
+      <c r="B142" s="5" t="inlineStr">
+        <is>
+          <t>Relative humidity at 08:30, Bengaluru</t>
+        </is>
+      </c>
+      <c r="C142" s="5" t="inlineStr">
+        <is>
+          <t>85 – 89</t>
+        </is>
+      </c>
+      <c r="D142" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E142" s="5" t="inlineStr">
+        <is>
+          <t>Monthly means, GKVK station</t>
+        </is>
+      </c>
+      <c r="F142" s="5" t="inlineStr">
+        <is>
+          <t>GKVK Bengaluru weather normals</t>
+        </is>
+      </c>
+      <c r="G142" s="5" t="inlineStr">
+        <is>
+          <t>University of Agricultural Sciences, Bangalore (GKVK agro-meteorological observatory) (n.d.). "Monthly weather normals, GKVK, Bengaluru". uasbangalore.edu.in.</t>
+        </is>
+      </c>
+      <c r="H142" s="5" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="I142" s="6" t="inlineStr">
+        <is>
+          <t>https://uasbangalore.edu.in/images/Agrometerology/pdf/gkvk-monthly-weather-normals-2011-2020-converted.pdf</t>
+        </is>
+      </c>
+      <c r="J142" s="5" t="inlineStr">
+        <is>
+          <t>Fusion study (doc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="5" t="n">
+        <v>119</v>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>Relative humidity at 17:30, Bengaluru</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>37 – 58</t>
+        </is>
+      </c>
+      <c r="D143" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E143" s="5" t="inlineStr">
+        <is>
+          <t>Monthly means (37 % Mar–Apr, 57–58 % Jul–Aug)</t>
+        </is>
+      </c>
+      <c r="F143" s="5" t="inlineStr">
+        <is>
+          <t>GKVK Bengaluru weather normals</t>
+        </is>
+      </c>
+      <c r="G143" s="5" t="inlineStr">
+        <is>
+          <t>University of Agricultural Sciences, Bangalore (GKVK agro-meteorological observatory) (n.d.). "Monthly weather normals, GKVK, Bengaluru". uasbangalore.edu.in.</t>
+        </is>
+      </c>
+      <c r="H143" s="5" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="I143" s="6" t="inlineStr">
+        <is>
+          <t>https://uasbangalore.edu.in/images/Agrometerology/pdf/gkvk-monthly-weather-normals-2011-2020-converted.pdf</t>
+        </is>
+      </c>
+      <c r="J143" s="5" t="inlineStr">
+        <is>
+          <t>Fusion study (doc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="5" t="n">
+        <v>120</v>
+      </c>
+      <c r="B144" s="5" t="inlineStr">
+        <is>
+          <t>Annual mean relative humidity at 17:30, Bengaluru</t>
+        </is>
+      </c>
+      <c r="C144" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="D144" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E144" s="5" t="inlineStr">
+        <is>
+          <t>GKVK station</t>
+        </is>
+      </c>
+      <c r="F144" s="5" t="inlineStr">
+        <is>
+          <t>GKVK Bengaluru weather normals</t>
+        </is>
+      </c>
+      <c r="G144" s="5" t="inlineStr">
+        <is>
+          <t>University of Agricultural Sciences, Bangalore (GKVK agro-meteorological observatory) (n.d.). "Monthly weather normals, GKVK, Bengaluru". uasbangalore.edu.in.</t>
+        </is>
+      </c>
+      <c r="H144" s="5" t="inlineStr">
+        <is>
+          <t>Table</t>
+        </is>
+      </c>
+      <c r="I144" s="6" t="inlineStr">
+        <is>
+          <t>https://uasbangalore.edu.in/images/Agrometerology/pdf/gkvk-monthly-weather-normals-2011-2020-converted.pdf</t>
+        </is>
+      </c>
+      <c r="J144" s="5" t="inlineStr">
+        <is>
+          <t>Fusion study (doc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>IPC ESD resource (ANSI/ESD S20.20)  —  electronics.org</t>
+        </is>
+      </c>
+      <c r="B145" s="3" t="n"/>
+      <c r="C145" s="3" t="n"/>
+      <c r="D145" s="3" t="n"/>
+      <c r="E145" s="3" t="n"/>
+      <c r="F145" s="3" t="n"/>
+      <c r="G145" s="3" t="n"/>
+      <c r="H145" s="3" t="n"/>
+      <c r="I145" s="3" t="n"/>
+      <c r="J145" s="4" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="5" t="n">
+        <v>121</v>
+      </c>
+      <c r="B146" s="5" t="inlineStr">
+        <is>
+          <t>Person-footwear-floor path limit in ESD areas</t>
+        </is>
+      </c>
+      <c r="C146" s="5" t="inlineStr">
+        <is>
+          <t>&lt; 1.0 × 10^9</t>
+        </is>
+      </c>
+      <c r="D146" s="5" t="inlineStr">
+        <is>
+          <t>Ω</t>
+        </is>
+      </c>
+      <c r="E146" s="5" t="inlineStr">
+        <is>
+          <t>ANSI/ESD S20.20; Ordinary shoes are far above this</t>
+        </is>
+      </c>
+      <c r="F146" s="5" t="inlineStr">
+        <is>
+          <t>IPC ESD resource (ANSI/ESD S20.20)</t>
+        </is>
+      </c>
+      <c r="G146" s="5" t="inlineStr">
+        <is>
+          <t>IPC (Electronics.org) technical resource (n.d.). "Electrostatic Discharge (ESD), Factory Issues, Measurement Methods". electronics.org.</t>
+        </is>
+      </c>
+      <c r="H146" s="5" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="I146" s="6" t="inlineStr">
+        <is>
+          <t>https://www.electronics.org/system/files/technical_resource/E15&amp;S22_02.pdf</t>
+        </is>
+      </c>
+      <c r="J146" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="5" t="n">
+        <v>122</v>
+      </c>
+      <c r="B147" s="5" t="inlineStr">
+        <is>
+          <t>ESD footwear resistance, low end</t>
+        </is>
+      </c>
+      <c r="C147" s="5" t="inlineStr">
+        <is>
+          <t>≈ 5 × 10^5</t>
+        </is>
+      </c>
+      <c r="D147" s="5" t="inlineStr">
+        <is>
+          <t>Ω</t>
+        </is>
+      </c>
+      <c r="E147" s="5" t="inlineStr">
+        <is>
+          <t>Commercial ESD footwear</t>
+        </is>
+      </c>
+      <c r="F147" s="5" t="inlineStr">
+        <is>
+          <t>IPC ESD resource (ANSI/ESD S20.20)</t>
+        </is>
+      </c>
+      <c r="G147" s="5" t="inlineStr">
+        <is>
+          <t>IPC (Electronics.org) technical resource (n.d.). "Electrostatic Discharge (ESD), Factory Issues, Measurement Methods". electronics.org.</t>
+        </is>
+      </c>
+      <c r="H147" s="5" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="I147" s="6" t="inlineStr">
+        <is>
+          <t>https://www.electronics.org/system/files/technical_resource/E15&amp;S22_02.pdf</t>
+        </is>
+      </c>
+      <c r="J147" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>Bian et al. 2025 (collaborative)  —  arXiv:2501.06940</t>
+        </is>
+      </c>
+      <c r="B148" s="3" t="n"/>
+      <c r="C148" s="3" t="n"/>
+      <c r="D148" s="3" t="n"/>
+      <c r="E148" s="3" t="n"/>
+      <c r="F148" s="3" t="n"/>
+      <c r="G148" s="3" t="n"/>
+      <c r="H148" s="3" t="n"/>
+      <c r="I148" s="3" t="n"/>
+      <c r="J148" s="4" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="5" t="n">
+        <v>123</v>
+      </c>
+      <c r="B149" s="5" t="inlineStr">
+        <is>
+          <t>Gain from adding body capacitance to wrist accelerometer (collaborative activities)</t>
+        </is>
+      </c>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>+16</t>
+        </is>
+      </c>
+      <c r="D149" s="5" t="inlineStr">
+        <is>
+          <t>% F-score</t>
+        </is>
+      </c>
+      <c r="E149" s="5" t="inlineStr">
+        <is>
+          <t>Collaborative activity recognition</t>
+        </is>
+      </c>
+      <c r="F149" s="5" t="inlineStr">
+        <is>
+          <t>Bian et al. 2025 (collaborative)</t>
+        </is>
+      </c>
+      <c r="G149" s="5" t="inlineStr">
+        <is>
+          <t>S. Bian, P. Lukowicz et al. (2025). "Collaborative Human Activity Recognition with Passive Inter-Body Electrostatic Field". arXiv:2501.06940.</t>
+        </is>
+      </c>
+      <c r="H149" s="5" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I149" s="6" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2501.06940</t>
+        </is>
+      </c>
+      <c r="J149" s="5" t="inlineStr">
+        <is>
+          <t>Accuracy benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>Bian et al. 2022 (leg motion)  —  Springer (book chapter)</t>
+        </is>
+      </c>
+      <c r="B150" s="3" t="n"/>
+      <c r="C150" s="3" t="n"/>
+      <c r="D150" s="3" t="n"/>
+      <c r="E150" s="3" t="n"/>
+      <c r="F150" s="3" t="n"/>
+      <c r="G150" s="3" t="n"/>
+      <c r="H150" s="3" t="n"/>
+      <c r="I150" s="3" t="n"/>
+      <c r="J150" s="4" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="5" t="n">
+        <v>124</v>
+      </c>
+      <c r="B151" s="5" t="inlineStr">
+        <is>
+          <t>Wrist body-capacitance vs IMU, leg-motion activities (F-score)</t>
+        </is>
+      </c>
+      <c r="C151" s="5" t="inlineStr">
+        <is>
+          <t>0.89 vs 0.78</t>
+        </is>
+      </c>
+      <c r="D151" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E151" s="5" t="inlineStr">
+        <is>
+          <t>Wrist-worn, leg-dominated activities</t>
+        </is>
+      </c>
+      <c r="F151" s="5" t="inlineStr">
+        <is>
+          <t>Bian et al. 2022 (leg motion)</t>
+        </is>
+      </c>
+      <c r="G151" s="5" t="inlineStr">
+        <is>
+          <t>S. Bian et al. (2022). "Using Human Body Capacitance Sensing to Monitor Leg Motion Dominated Activities with a Wrist Worn Device". Springer (book chapter).</t>
+        </is>
+      </c>
+      <c r="H151" s="5" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I151" s="6" t="inlineStr">
+        <is>
+          <t>https://link.springer.com/chapter/10.1007/978-981-19-0361-8_5</t>
+        </is>
+      </c>
+      <c r="J151" s="5" t="inlineStr">
+        <is>
+          <t>Accuracy benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>Loeffler 2014  —  PLOS ONE 9(9):e106664</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="n"/>
+      <c r="C152" s="3" t="n"/>
+      <c r="D152" s="3" t="n"/>
+      <c r="E152" s="3" t="n"/>
+      <c r="F152" s="3" t="n"/>
+      <c r="G152" s="3" t="n"/>
+      <c r="H152" s="3" t="n"/>
+      <c r="I152" s="3" t="n"/>
+      <c r="J152" s="4" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="5" t="n">
+        <v>125</v>
+      </c>
+      <c r="B153" s="5" t="inlineStr">
+        <is>
+          <t>Wrist accelerometer event detection accuracy (gunshot recoil)</t>
+        </is>
+      </c>
+      <c r="C153" s="5" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="D153" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E153" s="5" t="inlineStr">
+        <is>
+          <t>Hold-out set incl. confusable activities; Lab conditions</t>
+        </is>
+      </c>
+      <c r="F153" s="5" t="inlineStr">
+        <is>
+          <t>Loeffler 2014</t>
+        </is>
+      </c>
+      <c r="G153" s="5" t="inlineStr">
+        <is>
+          <t>C. E. Loeffler (2014). "Detecting Gunshots Using Wearable Accelerometers". PLOS ONE 9(9):e106664.</t>
+        </is>
+      </c>
+      <c r="H153" s="5" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I153" s="6" t="inlineStr">
+        <is>
+          <t>https://journals.plos.org/plosone/article?id=10.1371%2Fjournal.pone.0106664</t>
+        </is>
+      </c>
+      <c r="J153" s="5" t="inlineStr">
+        <is>
+          <t>Accuracy benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>Siirtola 2019  —  UbiComp/ISWC adjunct</t>
+        </is>
+      </c>
+      <c r="B154" s="3" t="n"/>
+      <c r="C154" s="3" t="n"/>
+      <c r="D154" s="3" t="n"/>
+      <c r="E154" s="3" t="n"/>
+      <c r="F154" s="3" t="n"/>
+      <c r="G154" s="3" t="n"/>
+      <c r="H154" s="3" t="n"/>
+      <c r="I154" s="3" t="n"/>
+      <c r="J154" s="4" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="5" t="n">
+        <v>126</v>
+      </c>
+      <c r="B155" s="5" t="inlineStr">
+        <is>
+          <t>Wrist-only stress detection, balanced accuracy</t>
+        </is>
+      </c>
+      <c r="C155" s="5" t="n">
+        <v>87.40000000000001</v>
+      </c>
+      <c r="D155" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E155" s="5" t="inlineStr">
+        <is>
+          <t>Empatica E4, WESAD, LDA</t>
+        </is>
+      </c>
+      <c r="F155" s="5" t="inlineStr">
+        <is>
+          <t>Siirtola 2019</t>
+        </is>
+      </c>
+      <c r="G155" s="5" t="inlineStr">
+        <is>
+          <t>P. Siirtola (2019). "Continuous stress detection using the sensors of commercial smartwatch (WESAD, Empatica E4)". UbiComp/ISWC adjunct.</t>
+        </is>
+      </c>
+      <c r="H155" s="5" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I155" s="6" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2203.09669</t>
+        </is>
+      </c>
+      <c r="J155" s="5" t="inlineStr">
+        <is>
+          <t>Accuracy benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>Schmidt et al. 2018 (WESAD)  —  ACM ICMI</t>
+        </is>
+      </c>
+      <c r="B156" s="3" t="n"/>
+      <c r="C156" s="3" t="n"/>
+      <c r="D156" s="3" t="n"/>
+      <c r="E156" s="3" t="n"/>
+      <c r="F156" s="3" t="n"/>
+      <c r="G156" s="3" t="n"/>
+      <c r="H156" s="3" t="n"/>
+      <c r="I156" s="3" t="n"/>
+      <c r="J156" s="4" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="5" t="n">
+        <v>127</v>
+      </c>
+      <c r="B157" s="5" t="inlineStr">
+        <is>
+          <t>Stress vs non-stress accuracy (best, chest device)</t>
+        </is>
+      </c>
+      <c r="C157" s="5" t="n">
+        <v>93</v>
+      </c>
+      <c r="D157" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E157" s="5" t="inlineStr">
+        <is>
+          <t>WESAD; Chest, not wrist</t>
+        </is>
+      </c>
+      <c r="F157" s="5" t="inlineStr">
+        <is>
+          <t>Schmidt et al. 2018 (WESAD)</t>
+        </is>
+      </c>
+      <c r="G157" s="5" t="inlineStr">
+        <is>
+          <t>P. Schmidt, A. Reiss, R. Duerichen, C. Marberger, K. Van Laerhoven (2018). "Introducing WESAD, a Multimodal Dataset for Wearable Stress and Affect Detection". ACM ICMI.</t>
+        </is>
+      </c>
+      <c r="H157" s="5" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I157" s="6" t="inlineStr">
+        <is>
+          <t>https://www.eti.uni-siegen.de/ubicomp/home/datasets/icmi18/</t>
+        </is>
+      </c>
+      <c r="J157" s="5" t="inlineStr">
+        <is>
+          <t>Accuracy benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>Audio distress detection 2026  —  arXiv:2608.04176</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="n"/>
+      <c r="C158" s="3" t="n"/>
+      <c r="D158" s="3" t="n"/>
+      <c r="E158" s="3" t="n"/>
+      <c r="F158" s="3" t="n"/>
+      <c r="G158" s="3" t="n"/>
+      <c r="H158" s="3" t="n"/>
+      <c r="I158" s="3" t="n"/>
+      <c r="J158" s="4" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="5" t="n">
+        <v>128</v>
+      </c>
+      <c r="B159" s="5" t="inlineStr">
+        <is>
+          <t>Scream stage false alarm rate, before / after context filter</t>
+        </is>
+      </c>
+      <c r="C159" s="5" t="inlineStr">
+        <is>
+          <t>≈ 10 / ≈ 1</t>
+        </is>
+      </c>
+      <c r="D159" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E159" s="5" t="inlineStr">
+        <is>
+          <t>Smartphone, daily audio; 1 % ≈ 15 min of false alarms per day</t>
+        </is>
+      </c>
+      <c r="F159" s="5" t="inlineStr">
+        <is>
+          <t>Audio distress detection 2026</t>
+        </is>
+      </c>
+      <c r="G159" s="5" t="inlineStr">
+        <is>
+          <t>(authors as listed on arXiv) (2026). "Smartphone Audio Based Distress Detection". arXiv:2608.04176.</t>
+        </is>
+      </c>
+      <c r="H159" s="5" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I159" s="6" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2608.04176</t>
+        </is>
+      </c>
+      <c r="J159" s="5" t="inlineStr">
+        <is>
+          <t>Accuracy benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>US Pat. 10,950,112  —  USPTO</t>
+        </is>
+      </c>
+      <c r="B160" s="3" t="n"/>
+      <c r="C160" s="3" t="n"/>
+      <c r="D160" s="3" t="n"/>
+      <c r="E160" s="3" t="n"/>
+      <c r="F160" s="3" t="n"/>
+      <c r="G160" s="3" t="n"/>
+      <c r="H160" s="3" t="n"/>
+      <c r="I160" s="3" t="n"/>
+      <c r="J160" s="4" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="5" t="n">
+        <v>129</v>
+      </c>
+      <c r="B161" s="5" t="inlineStr">
+        <is>
+          <t>Acceptable false-alarm budget for wrist detectors</t>
+        </is>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>≈ 1</t>
+        </is>
+      </c>
+      <c r="D161" s="5" t="inlineStr">
+        <is>
+          <t>per user per day</t>
+        </is>
+      </c>
+      <c r="E161" s="5" t="inlineStr">
+        <is>
+          <t>Stated as technically reasonable; many users find it too many; Patent text</t>
+        </is>
+      </c>
+      <c r="F161" s="5" t="inlineStr">
+        <is>
+          <t>US Pat. 10,950,112</t>
+        </is>
+      </c>
+      <c r="G161" s="5" t="inlineStr">
+        <is>
+          <t>US Patent 10,950,112 (n.d.). "Wrist fall detector based on arm direction". USPTO.</t>
+        </is>
+      </c>
+      <c r="H161" s="5" t="inlineStr">
+        <is>
+          <t>Background</t>
+        </is>
+      </c>
+      <c r="I161" s="6" t="inlineStr">
+        <is>
+          <t>https://image-ppubs.uspto.gov/dirsearch-public/print/downloadPdf/10950112</t>
+        </is>
+      </c>
+      <c r="J161" s="5" t="inlineStr">
+        <is>
+          <t>Accuracy benchmark</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J136"/>
-  <mergeCells count="22">
+  <autoFilter ref="A1:J161"/>
+  <mergeCells count="31">
+    <mergeCell ref="A160:J160"/>
     <mergeCell ref="A23:J23"/>
-    <mergeCell ref="A135:J135"/>
-    <mergeCell ref="A131:J131"/>
-    <mergeCell ref="A102:J102"/>
+    <mergeCell ref="A141:J141"/>
+    <mergeCell ref="A150:J150"/>
+    <mergeCell ref="A109:J109"/>
+    <mergeCell ref="A156:J156"/>
+    <mergeCell ref="A125:J125"/>
+    <mergeCell ref="A134:J134"/>
+    <mergeCell ref="A152:J152"/>
+    <mergeCell ref="A115:J115"/>
     <mergeCell ref="A31:J31"/>
-    <mergeCell ref="A127:J127"/>
-    <mergeCell ref="A114:J114"/>
+    <mergeCell ref="A148:J148"/>
     <mergeCell ref="A73:J73"/>
     <mergeCell ref="A98:J98"/>
     <mergeCell ref="A60:J60"/>
     <mergeCell ref="A49:J49"/>
+    <mergeCell ref="A138:J138"/>
+    <mergeCell ref="A103:J103"/>
+    <mergeCell ref="A132:J132"/>
     <mergeCell ref="A79:J79"/>
-    <mergeCell ref="A124:J124"/>
+    <mergeCell ref="A119:J119"/>
     <mergeCell ref="A90:J90"/>
-    <mergeCell ref="A108:J108"/>
+    <mergeCell ref="A128:J128"/>
     <mergeCell ref="A66:J66"/>
-    <mergeCell ref="A118:J118"/>
     <mergeCell ref="A37:J37"/>
-    <mergeCell ref="A133:J133"/>
+    <mergeCell ref="A145:J145"/>
+    <mergeCell ref="A158:J158"/>
+    <mergeCell ref="A136:J136"/>
+    <mergeCell ref="A154:J154"/>
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="A76:J76"/>
-    <mergeCell ref="A129:J129"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId1"/>
@@ -6516,31 +7459,47 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I99" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I100" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I101" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I103" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I102" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I104" r:id="rId90"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I105" r:id="rId91"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I106" r:id="rId92"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I107" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I109" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I108" r:id="rId94"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I110" r:id="rId95"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I111" r:id="rId96"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I112" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I113" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I115" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I114" r:id="rId99"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I116" r:id="rId100"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I117" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I119" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I118" r:id="rId102"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I120" r:id="rId103"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I121" r:id="rId104"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I122" r:id="rId105"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I123" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I125" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I124" r:id="rId107"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I126" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I128" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I130" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I132" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I134" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I136" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I127" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I129" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I130" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I131" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I133" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I135" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I137" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I139" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I140" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I142" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I143" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I144" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I146" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I147" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I149" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I151" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I153" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I155" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I157" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I159" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I161" r:id="rId129"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6552,7 +7511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6796,7 +7755,7 @@
         </is>
       </c>
       <c r="D13" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -6904,7 +7863,7 @@
         </is>
       </c>
       <c r="D19" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
@@ -6976,6 +7935,168 @@
         </is>
       </c>
       <c r="D23" s="8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>University of Agricultural Sciences, Bangalore (GKVK agro-meteorological observatory) (n.d.). "Monthly weather normals, GKVK, Bengaluru". uasbangalore.edu.in.</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>https://uasbangalore.edu.in/images/Agrometerology/pdf/gkvk-monthly-weather-normals-2011-2020-converted.pdf</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>IPC (Electronics.org) technical resource (n.d.). "Electrostatic Discharge (ESD), Factory Issues, Measurement Methods". electronics.org.</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>https://www.electronics.org/system/files/technical_resource/E15&amp;S22_02.pdf</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>S. Bian, P. Lukowicz et al. (2025). "Collaborative Human Activity Recognition with Passive Inter-Body Electrostatic Field". arXiv:2501.06940.</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2501.06940</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>S. Bian et al. (2022). "Using Human Body Capacitance Sensing to Monitor Leg Motion Dominated Activities with a Wrist Worn Device". Springer (book chapter).</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>https://link.springer.com/chapter/10.1007/978-981-19-0361-8_5</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>C. E. Loeffler (2014). "Detecting Gunshots Using Wearable Accelerometers". PLOS ONE 9(9):e106664.</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>https://journals.plos.org/plosone/article?id=10.1371%2Fjournal.pone.0106664</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>P. Siirtola (2019). "Continuous stress detection using the sensors of commercial smartwatch (WESAD, Empatica E4)". UbiComp/ISWC adjunct.</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2203.09669</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>P. Schmidt, A. Reiss, R. Duerichen, C. Marberger, K. Van Laerhoven (2018). "Introducing WESAD, a Multimodal Dataset for Wearable Stress and Affect Detection". ACM ICMI.</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>https://www.eti.uni-siegen.de/ubicomp/home/datasets/icmi18/</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>(authors as listed on arXiv) (2026). "Smartphone Audio Based Distress Detection". arXiv:2608.04176.</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2608.04176</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>US Patent 10,950,112 (n.d.). "Wrist fall detector based on arm direction". USPTO.</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>https://image-ppubs.uspto.gov/dirsearch-public/print/downloadPdf/10950112</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7003,6 +8124,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId31"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Replace estimates with published values (part 1): model, rates, passive physics, workbook
New sources S32-S58 logged in the paper-values workbook (165 values, 58 sources).
sg_model: sense-node parasitics from the OPA350 datasheet and PCB trace capacitance;
parylene coating permittivity. event_stream: watch-touch and phone rates and durations from
Visuri 2017 and Andrews 2015; walking body-capacitance swing from Ficker. sg_passive and the
demo sensor: cadence (Tudor-Locke), leak resistance range, one-foot capacitance and gait timing,
posture bound, wrist walking motion (Dawkins) and bus accelerations. SPICE cross-check and the
explorer port follow the new midpoints. Regenerated dataset, classifiers, figures, event stream.
</commit_message>
<xml_diff>
--- a/docs/SparshaGuard_paper_values.xlsx
+++ b/docs/SparshaGuard_paper_values.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference List" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Values from Papers'!$A$1:$J$161</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Values from Papers'!$A$1:$J$224</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J161"/>
+  <dimension ref="A1:J224"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7335,39 +7335,2266 @@
         </is>
       </c>
     </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>Talebzadeh et al. 2016  —  IEEE Trans. Electromagnetic Compatibility 58(4)</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="n"/>
+      <c r="C162" s="3" t="n"/>
+      <c r="D162" s="3" t="n"/>
+      <c r="E162" s="3" t="n"/>
+      <c r="F162" s="3" t="n"/>
+      <c r="G162" s="3" t="n"/>
+      <c r="H162" s="3" t="n"/>
+      <c r="I162" s="3" t="n"/>
+      <c r="J162" s="4" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="5" t="n">
+        <v>130</v>
+      </c>
+      <c r="B163" s="5" t="inlineStr">
+        <is>
+          <t>Body voltage, worst case (incl. walking)</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="inlineStr">
+        <is>
+          <t>&gt; ±20</t>
+        </is>
+      </c>
+      <c r="D163" s="5" t="inlineStr">
+        <is>
+          <t>kV</t>
+        </is>
+      </c>
+      <c r="E163" s="5" t="inlineStr">
+        <is>
+          <t>22 °C, 5 % RH</t>
+        </is>
+      </c>
+      <c r="F163" s="5" t="inlineStr">
+        <is>
+          <t>Talebzadeh et al. 2016</t>
+        </is>
+      </c>
+      <c r="G163" s="5" t="inlineStr">
+        <is>
+          <t>A. Talebzadeh, M. Moradian, Y. Han, D. E. Swenson, D. Pommerenke (2016). "Effect of Human Activities and Environmental Conditions on Electrostatic Charging". IEEE Trans. Electromagnetic Compatibility 58(4).</t>
+        </is>
+      </c>
+      <c r="H163" s="5" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I163" s="6" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/TEMC.2016.2575842</t>
+        </is>
+      </c>
+      <c r="J163" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="5" t="n">
+        <v>131</v>
+      </c>
+      <c r="B164" s="5" t="inlineStr">
+        <is>
+          <t>Body capacitance to ground on concrete vs wood-frame floor</t>
+        </is>
+      </c>
+      <c r="C164" s="5" t="inlineStr">
+        <is>
+          <t>120 vs 60</t>
+        </is>
+      </c>
+      <c r="D164" s="5" t="inlineStr">
+        <is>
+          <t>pF</t>
+        </is>
+      </c>
+      <c r="E164" s="5" t="inlineStr">
+        <is>
+          <t>Same person; concrete gives about half the voltage</t>
+        </is>
+      </c>
+      <c r="F164" s="5" t="inlineStr">
+        <is>
+          <t>Talebzadeh et al. 2016</t>
+        </is>
+      </c>
+      <c r="G164" s="5" t="inlineStr">
+        <is>
+          <t>A. Talebzadeh, M. Moradian, Y. Han, D. E. Swenson, D. Pommerenke (2016). "Effect of Human Activities and Environmental Conditions on Electrostatic Charging". IEEE Trans. Electromagnetic Compatibility 58(4).</t>
+        </is>
+      </c>
+      <c r="H164" s="5" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I164" s="6" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/TEMC.2016.2575842</t>
+        </is>
+      </c>
+      <c r="J164" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="5" t="n">
+        <v>132</v>
+      </c>
+      <c r="B165" s="5" t="inlineStr">
+        <is>
+          <t>Spread of body voltage from capacitance differences alone</t>
+        </is>
+      </c>
+      <c r="C165" s="5" t="inlineStr">
+        <is>
+          <t>±30</t>
+        </is>
+      </c>
+      <c r="D165" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E165" s="5" t="inlineStr"/>
+      <c r="F165" s="5" t="inlineStr">
+        <is>
+          <t>Talebzadeh et al. 2016</t>
+        </is>
+      </c>
+      <c r="G165" s="5" t="inlineStr">
+        <is>
+          <t>A. Talebzadeh, M. Moradian, Y. Han, D. E. Swenson, D. Pommerenke (2016). "Effect of Human Activities and Environmental Conditions on Electrostatic Charging". IEEE Trans. Electromagnetic Compatibility 58(4).</t>
+        </is>
+      </c>
+      <c r="H165" s="5" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I165" s="6" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/TEMC.2016.2575842</t>
+        </is>
+      </c>
+      <c r="J165" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="5" t="n">
+        <v>133</v>
+      </c>
+      <c r="B166" s="5" t="inlineStr">
+        <is>
+          <t>Time for body charge to fall to 100 V without ESD shoes/floor</t>
+        </is>
+      </c>
+      <c r="C166" s="5" t="inlineStr">
+        <is>
+          <t>1 – 30</t>
+        </is>
+      </c>
+      <c r="D166" s="5" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="E166" s="5" t="inlineStr">
+        <is>
+          <t>With ESD shoes/floor: 0.5–6 s</t>
+        </is>
+      </c>
+      <c r="F166" s="5" t="inlineStr">
+        <is>
+          <t>Talebzadeh et al. 2016</t>
+        </is>
+      </c>
+      <c r="G166" s="5" t="inlineStr">
+        <is>
+          <t>A. Talebzadeh, M. Moradian, Y. Han, D. E. Swenson, D. Pommerenke (2016). "Effect of Human Activities and Environmental Conditions on Electrostatic Charging". IEEE Trans. Electromagnetic Compatibility 58(4).</t>
+        </is>
+      </c>
+      <c r="H166" s="5" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I166" s="6" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/TEMC.2016.2575842</t>
+        </is>
+      </c>
+      <c r="J166" s="5" t="inlineStr">
+        <is>
+          <t>Yes (in model, Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>Kangas et al. 2015  —  Gerontology 61(1):61-68</t>
+        </is>
+      </c>
+      <c r="B167" s="3" t="n"/>
+      <c r="C167" s="3" t="n"/>
+      <c r="D167" s="3" t="n"/>
+      <c r="E167" s="3" t="n"/>
+      <c r="F167" s="3" t="n"/>
+      <c r="G167" s="3" t="n"/>
+      <c r="H167" s="3" t="n"/>
+      <c r="I167" s="3" t="n"/>
+      <c r="J167" s="4" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="5" t="n">
+        <v>134</v>
+      </c>
+      <c r="B168" s="5" t="inlineStr">
+        <is>
+          <t>Fall-sensor false alarms in long-term use</t>
+        </is>
+      </c>
+      <c r="C168" s="5" t="inlineStr">
+        <is>
+          <t>0.049 (0.025 improved)</t>
+        </is>
+      </c>
+      <c r="D168" s="5" t="inlineStr">
+        <is>
+          <t>per hour</t>
+        </is>
+      </c>
+      <c r="E168" s="5" t="inlineStr">
+        <is>
+          <t>16 older adults, 15,500 h</t>
+        </is>
+      </c>
+      <c r="F168" s="5" t="inlineStr">
+        <is>
+          <t>Kangas et al. 2015</t>
+        </is>
+      </c>
+      <c r="G168" s="5" t="inlineStr">
+        <is>
+          <t>M. Kangas, R. Korpelainen, I. Vikman, L. Nyberg, T. Jämsä (2015). "Sensitivity and false alarm rate of a fall sensor in long-term fall detection in the elderly". Gerontology 61(1):61-68.</t>
+        </is>
+      </c>
+      <c r="H168" s="5" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I168" s="6" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1159/000362720</t>
+        </is>
+      </c>
+      <c r="J168" s="5" t="inlineStr">
+        <is>
+          <t>Accuracy benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>Tchuente et al. 2020  —  Sensors 20(21):6377</t>
+        </is>
+      </c>
+      <c r="B169" s="3" t="n"/>
+      <c r="C169" s="3" t="n"/>
+      <c r="D169" s="3" t="n"/>
+      <c r="E169" s="3" t="n"/>
+      <c r="F169" s="3" t="n"/>
+      <c r="G169" s="3" t="n"/>
+      <c r="H169" s="3" t="n"/>
+      <c r="I169" s="3" t="n"/>
+      <c r="J169" s="4" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="5" t="n">
+        <v>135</v>
+      </c>
+      <c r="B170" s="5" t="inlineStr">
+        <is>
+          <t>Aggressive-movement classification, smartwatch</t>
+        </is>
+      </c>
+      <c r="C170" s="5" t="inlineStr">
+        <is>
+          <t>99.6 % accuracy, 98.4 % sensitivity</t>
+        </is>
+      </c>
+      <c r="D170" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E170" s="5" t="inlineStr">
+        <is>
+          <t>30 people, scripted punch/shove/slap; Scripted</t>
+        </is>
+      </c>
+      <c r="F170" s="5" t="inlineStr">
+        <is>
+          <t>Tchuente et al. 2020</t>
+        </is>
+      </c>
+      <c r="G170" s="5" t="inlineStr">
+        <is>
+          <t>F. Tchuente, N. Baddour, E. D. Lemaire (2020). "Classification of Aggressive Movements Using Smartwatches". Sensors 20(21):6377.</t>
+        </is>
+      </c>
+      <c r="H170" s="5" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I170" s="6" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/s20216377</t>
+        </is>
+      </c>
+      <c r="J170" s="5" t="inlineStr">
+        <is>
+          <t>Accuracy benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>TI OPA350 datasheet  —  Datasheet</t>
+        </is>
+      </c>
+      <c r="B171" s="3" t="n"/>
+      <c r="C171" s="3" t="n"/>
+      <c r="D171" s="3" t="n"/>
+      <c r="E171" s="3" t="n"/>
+      <c r="F171" s="3" t="n"/>
+      <c r="G171" s="3" t="n"/>
+      <c r="H171" s="3" t="n"/>
+      <c r="I171" s="3" t="n"/>
+      <c r="J171" s="4" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="5" t="n">
+        <v>136</v>
+      </c>
+      <c r="B172" s="5" t="inlineStr">
+        <is>
+          <t>OPA350 input capacitance</t>
+        </is>
+      </c>
+      <c r="C172" s="5" t="inlineStr">
+        <is>
+          <t>≈ 9</t>
+        </is>
+      </c>
+      <c r="D172" s="5" t="inlineStr">
+        <is>
+          <t>pF</t>
+        </is>
+      </c>
+      <c r="E172" s="5" t="inlineStr">
+        <is>
+          <t>Typical</t>
+        </is>
+      </c>
+      <c r="F172" s="5" t="inlineStr">
+        <is>
+          <t>TI OPA350 datasheet</t>
+        </is>
+      </c>
+      <c r="G172" s="5" t="inlineStr">
+        <is>
+          <t>Texas Instruments (2015). "OPA350, OPA2350, OPA4350 high-speed single-supply rail-to-rail operational amplifiers (SBOS099D)". Datasheet.</t>
+        </is>
+      </c>
+      <c r="H172" s="5" t="inlineStr">
+        <is>
+          <t>Datasheet</t>
+        </is>
+      </c>
+      <c r="I172" s="6" t="inlineStr">
+        <is>
+          <t>https://www.ti.com/lit/ds/symlink/opa350.pdf</t>
+        </is>
+      </c>
+      <c r="J172" s="5" t="inlineStr">
+        <is>
+          <t>Yes (in model, Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>ECN trace capacitance  —  Trade article</t>
+        </is>
+      </c>
+      <c r="B173" s="3" t="n"/>
+      <c r="C173" s="3" t="n"/>
+      <c r="D173" s="3" t="n"/>
+      <c r="E173" s="3" t="n"/>
+      <c r="F173" s="3" t="n"/>
+      <c r="G173" s="3" t="n"/>
+      <c r="H173" s="3" t="n"/>
+      <c r="I173" s="3" t="n"/>
+      <c r="J173" s="4" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="5" t="n">
+        <v>137</v>
+      </c>
+      <c r="B174" s="5" t="inlineStr">
+        <is>
+          <t>PCB trace capacitance</t>
+        </is>
+      </c>
+      <c r="C174" s="5" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D174" s="5" t="inlineStr">
+        <is>
+          <t>pF/cm</t>
+        </is>
+      </c>
+      <c r="E174" s="5" t="inlineStr">
+        <is>
+          <t>0.8 mm trace on 0.8 mm FR-4 over a plane</t>
+        </is>
+      </c>
+      <c r="F174" s="5" t="inlineStr">
+        <is>
+          <t>ECN trace capacitance</t>
+        </is>
+      </c>
+      <c r="G174" s="5" t="inlineStr">
+        <is>
+          <t>ECN / passive-components.eu (using TI figures) (n.d.). "A Plague of Parasites (PCB trace capacitance)". Trade article.</t>
+        </is>
+      </c>
+      <c r="H174" s="5" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="I174" s="6" t="inlineStr">
+        <is>
+          <t>https://passive-components.eu/</t>
+        </is>
+      </c>
+      <c r="J174" s="5" t="inlineStr">
+        <is>
+          <t>Yes (in model, Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>SCS parylene data  —  Manufacturer technical data</t>
+        </is>
+      </c>
+      <c r="B175" s="3" t="n"/>
+      <c r="C175" s="3" t="n"/>
+      <c r="D175" s="3" t="n"/>
+      <c r="E175" s="3" t="n"/>
+      <c r="F175" s="3" t="n"/>
+      <c r="G175" s="3" t="n"/>
+      <c r="H175" s="3" t="n"/>
+      <c r="I175" s="3" t="n"/>
+      <c r="J175" s="4" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="5" t="n">
+        <v>138</v>
+      </c>
+      <c r="B176" s="5" t="inlineStr">
+        <is>
+          <t>Parylene relative permittivity, N / C</t>
+        </is>
+      </c>
+      <c r="C176" s="5" t="inlineStr">
+        <is>
+          <t>2.65 / 2.95–3.15</t>
+        </is>
+      </c>
+      <c r="D176" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E176" s="5" t="inlineStr">
+        <is>
+          <t>1 MHz (C: 3.15 at 60 Hz)</t>
+        </is>
+      </c>
+      <c r="F176" s="5" t="inlineStr">
+        <is>
+          <t>SCS parylene data</t>
+        </is>
+      </c>
+      <c r="G176" s="5" t="inlineStr">
+        <is>
+          <t>Specialty Coating Systems (n.d.). "Parylene Dielectric Properties". Manufacturer technical data.</t>
+        </is>
+      </c>
+      <c r="H176" s="5" t="inlineStr">
+        <is>
+          <t>Data sheet</t>
+        </is>
+      </c>
+      <c r="I176" s="6" t="inlineStr">
+        <is>
+          <t>https://scscoatings.com/</t>
+        </is>
+      </c>
+      <c r="J176" s="5" t="inlineStr">
+        <is>
+          <t>Yes (in model, Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>Visuri et al. 2017  —  Proc. ACM CHI 2017, pp. 3569-3581</t>
+        </is>
+      </c>
+      <c r="B177" s="3" t="n"/>
+      <c r="C177" s="3" t="n"/>
+      <c r="D177" s="3" t="n"/>
+      <c r="E177" s="3" t="n"/>
+      <c r="F177" s="3" t="n"/>
+      <c r="G177" s="3" t="n"/>
+      <c r="H177" s="3" t="n"/>
+      <c r="I177" s="3" t="n"/>
+      <c r="J177" s="4" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="5" t="n">
+        <v>139</v>
+      </c>
+      <c r="B178" s="5" t="inlineStr">
+        <is>
+          <t>Smartwatch usage sessions</t>
+        </is>
+      </c>
+      <c r="C178" s="5" t="inlineStr">
+        <is>
+          <t>≈ 140</t>
+        </is>
+      </c>
+      <c r="D178" s="5" t="inlineStr">
+        <is>
+          <t>per day</t>
+        </is>
+      </c>
+      <c r="E178" s="5" t="inlineStr">
+        <is>
+          <t>307 users; about two-thirds are glances; 140/day secondary</t>
+        </is>
+      </c>
+      <c r="F178" s="5" t="inlineStr">
+        <is>
+          <t>Visuri et al. 2017</t>
+        </is>
+      </c>
+      <c r="G178" s="5" t="inlineStr">
+        <is>
+          <t>A. Visuri, Z. Sarsenbayeva, N. van Berkel, J. Goncalves, R. Rawassizadeh, V. Kostakos, D. Ferreira (2017). "Quantifying Sources and Types of Smartwatch Usage Sessions". Proc. ACM CHI 2017, pp. 3569-3581.</t>
+        </is>
+      </c>
+      <c r="H178" s="5" t="inlineStr">
+        <is>
+          <t>Abstract + news</t>
+        </is>
+      </c>
+      <c r="I178" s="6" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1145/3025453.3025817</t>
+        </is>
+      </c>
+      <c r="J178" s="5" t="inlineStr">
+        <is>
+          <t>Yes (in model, Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="5" t="n">
+        <v>140</v>
+      </c>
+      <c r="B179" s="5" t="inlineStr">
+        <is>
+          <t>Smartwatch sessions shorter than 5 s; mean session</t>
+        </is>
+      </c>
+      <c r="C179" s="5" t="inlineStr">
+        <is>
+          <t>half; ≈ 9 s</t>
+        </is>
+      </c>
+      <c r="D179" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E179" s="5" t="inlineStr"/>
+      <c r="F179" s="5" t="inlineStr">
+        <is>
+          <t>Visuri et al. 2017</t>
+        </is>
+      </c>
+      <c r="G179" s="5" t="inlineStr">
+        <is>
+          <t>A. Visuri, Z. Sarsenbayeva, N. van Berkel, J. Goncalves, R. Rawassizadeh, V. Kostakos, D. Ferreira (2017). "Quantifying Sources and Types of Smartwatch Usage Sessions". Proc. ACM CHI 2017, pp. 3569-3581.</t>
+        </is>
+      </c>
+      <c r="H179" s="5" t="inlineStr">
+        <is>
+          <t>Abstract + news</t>
+        </is>
+      </c>
+      <c r="I179" s="6" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1145/3025453.3025817</t>
+        </is>
+      </c>
+      <c r="J179" s="5" t="inlineStr">
+        <is>
+          <t>Yes (in model, Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>Andrews et al. 2015  —  PLoS ONE 10(10):e0139004</t>
+        </is>
+      </c>
+      <c r="B180" s="3" t="n"/>
+      <c r="C180" s="3" t="n"/>
+      <c r="D180" s="3" t="n"/>
+      <c r="E180" s="3" t="n"/>
+      <c r="F180" s="3" t="n"/>
+      <c r="G180" s="3" t="n"/>
+      <c r="H180" s="3" t="n"/>
+      <c r="I180" s="3" t="n"/>
+      <c r="J180" s="4" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="5" t="n">
+        <v>141</v>
+      </c>
+      <c r="B181" s="5" t="inlineStr">
+        <is>
+          <t>Smartphone uses per day; total use</t>
+        </is>
+      </c>
+      <c r="C181" s="5" t="inlineStr">
+        <is>
+          <t>≈ 85; ≈ 5 h</t>
+        </is>
+      </c>
+      <c r="D181" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E181" s="5" t="inlineStr">
+        <is>
+          <t>23 adults, 2 weeks; more than half under 30 s; Secondary</t>
+        </is>
+      </c>
+      <c r="F181" s="5" t="inlineStr">
+        <is>
+          <t>Andrews et al. 2015</t>
+        </is>
+      </c>
+      <c r="G181" s="5" t="inlineStr">
+        <is>
+          <t>S. Andrews, D. A. Ellis, H. Shaw, L. Piwek (2015). "Beyond Self-Report: Tools to Compare Estimated and Real-World Smartphone Use". PLoS ONE 10(10):e0139004.</t>
+        </is>
+      </c>
+      <c r="H181" s="5" t="inlineStr">
+        <is>
+          <t>Press release</t>
+        </is>
+      </c>
+      <c r="I181" s="6" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1371/journal.pone.0139004</t>
+        </is>
+      </c>
+      <c r="J181" s="5" t="inlineStr">
+        <is>
+          <t>Yes (in model, Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>Ficker 2005  —  J. Phys. D: Appl. Phys. 38(5):410-417</t>
+        </is>
+      </c>
+      <c r="B182" s="3" t="n"/>
+      <c r="C182" s="3" t="n"/>
+      <c r="D182" s="3" t="n"/>
+      <c r="E182" s="3" t="n"/>
+      <c r="F182" s="3" t="n"/>
+      <c r="G182" s="3" t="n"/>
+      <c r="H182" s="3" t="n"/>
+      <c r="I182" s="3" t="n"/>
+      <c r="J182" s="4" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="5" t="n">
+        <v>142</v>
+      </c>
+      <c r="B183" s="5" t="inlineStr">
+        <is>
+          <t>Body capacitance standing on both feet / on one foot</t>
+        </is>
+      </c>
+      <c r="C183" s="5" t="inlineStr">
+        <is>
+          <t>160 / 100</t>
+        </is>
+      </c>
+      <c r="D183" s="5" t="inlineStr">
+        <is>
+          <t>pF</t>
+        </is>
+      </c>
+      <c r="E183" s="5" t="inlineStr">
+        <is>
+          <t>Vinyl tile; Secondary</t>
+        </is>
+      </c>
+      <c r="F183" s="5" t="inlineStr">
+        <is>
+          <t>Ficker 2005</t>
+        </is>
+      </c>
+      <c r="G183" s="5" t="inlineStr">
+        <is>
+          <t>T. Ficker (2005). "Charging by walking". J. Phys. D: Appl. Phys. 38(5):410-417.</t>
+        </is>
+      </c>
+      <c r="H183" s="5" t="inlineStr">
+        <is>
+          <t>Summary article</t>
+        </is>
+      </c>
+      <c r="I183" s="6" t="inlineStr">
+        <is>
+          <t>https://incompliancemag.com/charging-by-walking/</t>
+        </is>
+      </c>
+      <c r="J183" s="5" t="inlineStr">
+        <is>
+          <t>Yes (in model, Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="5" t="n">
+        <v>143</v>
+      </c>
+      <c r="B184" s="5" t="inlineStr">
+        <is>
+          <t>Body resistance to ground on vinyl tile</t>
+        </is>
+      </c>
+      <c r="C184" s="5" t="inlineStr">
+        <is>
+          <t>≈ 10^11</t>
+        </is>
+      </c>
+      <c r="D184" s="5" t="inlineStr">
+        <is>
+          <t>Ω</t>
+        </is>
+      </c>
+      <c r="E184" s="5" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="F184" s="5" t="inlineStr">
+        <is>
+          <t>Ficker 2005</t>
+        </is>
+      </c>
+      <c r="G184" s="5" t="inlineStr">
+        <is>
+          <t>T. Ficker (2005). "Charging by walking". J. Phys. D: Appl. Phys. 38(5):410-417.</t>
+        </is>
+      </c>
+      <c r="H184" s="5" t="inlineStr">
+        <is>
+          <t>Summary article</t>
+        </is>
+      </c>
+      <c r="I184" s="6" t="inlineStr">
+        <is>
+          <t>https://incompliancemag.com/charging-by-walking/</t>
+        </is>
+      </c>
+      <c r="J184" s="5" t="inlineStr">
+        <is>
+          <t>Yes (in model, Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="5" t="n">
+        <v>144</v>
+      </c>
+      <c r="B185" s="5" t="inlineStr">
+        <is>
+          <t>Lifting a foot raises body voltage</t>
+        </is>
+      </c>
+      <c r="C185" s="5" t="inlineStr">
+        <is>
+          <t>8 – 12</t>
+        </is>
+      </c>
+      <c r="D185" s="5" t="inlineStr">
+        <is>
+          <t>×</t>
+        </is>
+      </c>
+      <c r="E185" s="5" t="inlineStr">
+        <is>
+          <t>Walking on resistive floors; Secondary</t>
+        </is>
+      </c>
+      <c r="F185" s="5" t="inlineStr">
+        <is>
+          <t>Ficker 2005</t>
+        </is>
+      </c>
+      <c r="G185" s="5" t="inlineStr">
+        <is>
+          <t>T. Ficker (2005). "Charging by walking". J. Phys. D: Appl. Phys. 38(5):410-417.</t>
+        </is>
+      </c>
+      <c r="H185" s="5" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="I185" s="6" t="inlineStr">
+        <is>
+          <t>https://incompliancemag.com/charging-by-walking/</t>
+        </is>
+      </c>
+      <c r="J185" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>Tudor-Locke et al. 2012  —  Sports Medicine 42(5):381-398</t>
+        </is>
+      </c>
+      <c r="B186" s="3" t="n"/>
+      <c r="C186" s="3" t="n"/>
+      <c r="D186" s="3" t="n"/>
+      <c r="E186" s="3" t="n"/>
+      <c r="F186" s="3" t="n"/>
+      <c r="G186" s="3" t="n"/>
+      <c r="H186" s="3" t="n"/>
+      <c r="I186" s="3" t="n"/>
+      <c r="J186" s="4" t="n"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="5" t="n">
+        <v>145</v>
+      </c>
+      <c r="B187" s="5" t="inlineStr">
+        <is>
+          <t>Walking cadence, women (normal lab walking)</t>
+        </is>
+      </c>
+      <c r="C187" s="5" t="inlineStr">
+        <is>
+          <t>96 – 138</t>
+        </is>
+      </c>
+      <c r="D187" s="5" t="inlineStr">
+        <is>
+          <t>steps/min</t>
+        </is>
+      </c>
+      <c r="E187" s="5" t="inlineStr">
+        <is>
+          <t>Across the lifespan</t>
+        </is>
+      </c>
+      <c r="F187" s="5" t="inlineStr">
+        <is>
+          <t>Tudor-Locke et al. 2012</t>
+        </is>
+      </c>
+      <c r="G187" s="5" t="inlineStr">
+        <is>
+          <t>C. Tudor-Locke, H. Han, E. J. Aguiar, et al. (2012). "Using cadence to study free-living ambulatory activity". Sports Medicine 42(5):381-398.</t>
+        </is>
+      </c>
+      <c r="H187" s="5" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I187" s="6" t="inlineStr">
+        <is>
+          <t>https://strathprints.strath.ac.uk/42646/</t>
+        </is>
+      </c>
+      <c r="J187" s="5" t="inlineStr">
+        <is>
+          <t>Yes (in model, Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>Neacsu et al. 2007  —  IMEKO TC4 Symposium, Iasi</t>
+        </is>
+      </c>
+      <c r="B188" s="3" t="n"/>
+      <c r="C188" s="3" t="n"/>
+      <c r="D188" s="3" t="n"/>
+      <c r="E188" s="3" t="n"/>
+      <c r="F188" s="3" t="n"/>
+      <c r="G188" s="3" t="n"/>
+      <c r="H188" s="3" t="n"/>
+      <c r="I188" s="3" t="n"/>
+      <c r="J188" s="4" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="5" t="n">
+        <v>146</v>
+      </c>
+      <c r="B189" s="5" t="inlineStr">
+        <is>
+          <t>Change of body capacitance, sitting on a wooden chair vs standing</t>
+        </is>
+      </c>
+      <c r="C189" s="5" t="inlineStr">
+        <is>
+          <t>&lt; 10</t>
+        </is>
+      </c>
+      <c r="D189" s="5" t="inlineStr">
+        <is>
+          <t>pF</t>
+        </is>
+      </c>
+      <c r="E189" s="5" t="inlineStr"/>
+      <c r="F189" s="5" t="inlineStr">
+        <is>
+          <t>Neacsu et al. 2007</t>
+        </is>
+      </c>
+      <c r="G189" s="5" t="inlineStr">
+        <is>
+          <t>D. Neacsu, A. Salceanu, E. Lunca, V. David (2007). "Indirect Measurements on the Capacity in the Electrostatic HB Model". IMEKO TC4 Symposium, Iasi.</t>
+        </is>
+      </c>
+      <c r="H189" s="5" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I189" s="6" t="inlineStr">
+        <is>
+          <t>https://imeko.org/proceedings/indirect-measurements-on-the-capacity-in-the-electrostatic-hb-model</t>
+        </is>
+      </c>
+      <c r="J189" s="5" t="inlineStr">
+        <is>
+          <t>Yes (in model, Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="5" t="n">
+        <v>147</v>
+      </c>
+      <c r="B190" s="5" t="inlineStr">
+        <is>
+          <t>Measured human body capacitance, range</t>
+        </is>
+      </c>
+      <c r="C190" s="5" t="inlineStr">
+        <is>
+          <t>50 – 500</t>
+        </is>
+      </c>
+      <c r="D190" s="5" t="inlineStr">
+        <is>
+          <t>pF</t>
+        </is>
+      </c>
+      <c r="E190" s="5" t="inlineStr"/>
+      <c r="F190" s="5" t="inlineStr">
+        <is>
+          <t>Neacsu et al. 2007</t>
+        </is>
+      </c>
+      <c r="G190" s="5" t="inlineStr">
+        <is>
+          <t>D. Neacsu, A. Salceanu, E. Lunca, V. David (2007). "Indirect Measurements on the Capacity in the Electrostatic HB Model". IMEKO TC4 Symposium, Iasi.</t>
+        </is>
+      </c>
+      <c r="H190" s="5" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I190" s="6" t="inlineStr">
+        <is>
+          <t>https://imeko.org/proceedings/indirect-measurements-on-the-capacity-in-the-electrostatic-hb-model</t>
+        </is>
+      </c>
+      <c r="J190" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="5" t="n">
+        <v>148</v>
+      </c>
+      <c r="B191" s="5" t="inlineStr">
+        <is>
+          <t>Body capacitance barefoot on 1 rubber carpet / on 4 carpets</t>
+        </is>
+      </c>
+      <c r="C191" s="5" t="inlineStr">
+        <is>
+          <t>295 / 116</t>
+        </is>
+      </c>
+      <c r="D191" s="5" t="inlineStr">
+        <is>
+          <t>pF</t>
+        </is>
+      </c>
+      <c r="E191" s="5" t="inlineStr"/>
+      <c r="F191" s="5" t="inlineStr">
+        <is>
+          <t>Neacsu et al. 2007</t>
+        </is>
+      </c>
+      <c r="G191" s="5" t="inlineStr">
+        <is>
+          <t>D. Neacsu, A. Salceanu, E. Lunca, V. David (2007). "Indirect Measurements on the Capacity in the Electrostatic HB Model". IMEKO TC4 Symposium, Iasi.</t>
+        </is>
+      </c>
+      <c r="H191" s="5" t="inlineStr">
+        <is>
+          <t>Snippet</t>
+        </is>
+      </c>
+      <c r="I191" s="6" t="inlineStr">
+        <is>
+          <t>https://imeko.org/proceedings/indirect-measurements-on-the-capacity-in-the-electrostatic-hb-model</t>
+        </is>
+      </c>
+      <c r="J191" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>Dawkins et al. 2022  —  J. Sports Sciences</t>
+        </is>
+      </c>
+      <c r="B192" s="3" t="n"/>
+      <c r="C192" s="3" t="n"/>
+      <c r="D192" s="3" t="n"/>
+      <c r="E192" s="3" t="n"/>
+      <c r="F192" s="3" t="n"/>
+      <c r="G192" s="3" t="n"/>
+      <c r="H192" s="3" t="n"/>
+      <c r="I192" s="3" t="n"/>
+      <c r="J192" s="4" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="5" t="n">
+        <v>149</v>
+      </c>
+      <c r="B193" s="5" t="inlineStr">
+        <is>
+          <t>Wrist acceleration (ENMO), slow / normal / brisk walking</t>
+        </is>
+      </c>
+      <c r="C193" s="5" t="inlineStr">
+        <is>
+          <t>140 / 210 / 350</t>
+        </is>
+      </c>
+      <c r="D193" s="5" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="E193" s="5" t="inlineStr">
+        <is>
+          <t>Adults 40–69, wrist, averaged; Averaged, not peaks</t>
+        </is>
+      </c>
+      <c r="F193" s="5" t="inlineStr">
+        <is>
+          <t>Dawkins et al. 2022</t>
+        </is>
+      </c>
+      <c r="G193" s="5" t="inlineStr">
+        <is>
+          <t>N. P. Dawkins, T. Yates, et al. (2022). "Normative wrist-worn accelerometer values for self-paced walking and running: a walk in the park". J. Sports Sciences.</t>
+        </is>
+      </c>
+      <c r="H193" s="5" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I193" s="6" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1080/02640414.2021.1976491</t>
+        </is>
+      </c>
+      <c r="J193" s="5" t="inlineStr">
+        <is>
+          <t>Yes (in model, Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>Walking recognition 2022  —  arXiv:2207.07443</t>
+        </is>
+      </c>
+      <c r="B194" s="3" t="n"/>
+      <c r="C194" s="3" t="n"/>
+      <c r="D194" s="3" t="n"/>
+      <c r="E194" s="3" t="n"/>
+      <c r="F194" s="3" t="n"/>
+      <c r="G194" s="3" t="n"/>
+      <c r="H194" s="3" t="n"/>
+      <c r="I194" s="3" t="n"/>
+      <c r="J194" s="4" t="n"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="5" t="n">
+        <v>150</v>
+      </c>
+      <c r="B195" s="5" t="inlineStr">
+        <is>
+          <t>Walking periodicity; wrist shows half the step rate</t>
+        </is>
+      </c>
+      <c r="C195" s="5" t="inlineStr">
+        <is>
+          <t>≈ 1.7</t>
+        </is>
+      </c>
+      <c r="D195" s="5" t="inlineStr">
+        <is>
+          <t>Hz</t>
+        </is>
+      </c>
+      <c r="E195" s="5" t="inlineStr">
+        <is>
+          <t>Pooled datasets</t>
+        </is>
+      </c>
+      <c r="F195" s="5" t="inlineStr">
+        <is>
+          <t>Walking recognition 2022</t>
+        </is>
+      </c>
+      <c r="G195" s="5" t="inlineStr">
+        <is>
+          <t>(authors as listed on arXiv) (2022). "A 'one-size-fits-most' walking recognition method for smartphones, smartwatches, and wearable accelerometers". arXiv:2207.07443.</t>
+        </is>
+      </c>
+      <c r="H195" s="5" t="inlineStr">
+        <is>
+          <t>Snippet</t>
+        </is>
+      </c>
+      <c r="I195" s="6" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2207.07443</t>
+        </is>
+      </c>
+      <c r="J195" s="5" t="inlineStr">
+        <is>
+          <t>Yes (in model, Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>Public transport perturbation 2020  —  Z. Gerontol. Geriatr.</t>
+        </is>
+      </c>
+      <c r="B196" s="3" t="n"/>
+      <c r="C196" s="3" t="n"/>
+      <c r="D196" s="3" t="n"/>
+      <c r="E196" s="3" t="n"/>
+      <c r="F196" s="3" t="n"/>
+      <c r="G196" s="3" t="n"/>
+      <c r="H196" s="3" t="n"/>
+      <c r="I196" s="3" t="n"/>
+      <c r="J196" s="4" t="n"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="5" t="n">
+        <v>151</v>
+      </c>
+      <c r="B197" s="5" t="inlineStr">
+        <is>
+          <t>Bus acceleration from standstill / braking into a stop, maxima</t>
+        </is>
+      </c>
+      <c r="C197" s="5" t="inlineStr">
+        <is>
+          <t>3.37 / −3.12</t>
+        </is>
+      </c>
+      <c r="D197" s="5" t="inlineStr">
+        <is>
+          <t>m/s²</t>
+        </is>
+      </c>
+      <c r="E197" s="5" t="inlineStr">
+        <is>
+          <t>12 days, sensor on a vertical bar</t>
+        </is>
+      </c>
+      <c r="F197" s="5" t="inlineStr">
+        <is>
+          <t>Public transport perturbation 2020</t>
+        </is>
+      </c>
+      <c r="G197" s="5" t="inlineStr">
+        <is>
+          <t>(authors not visible in the abstract) (2020). "Perturbation in public transport as a basic concept for perturbation-based balance training for fall prevention". Z. Gerontol. Geriatr..</t>
+        </is>
+      </c>
+      <c r="H197" s="5" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I197" s="6" t="inlineStr">
+        <is>
+          <t>https://link.springer.com/journal/391</t>
+        </is>
+      </c>
+      <c r="J197" s="5" t="inlineStr">
+        <is>
+          <t>Yes (in model, Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="5" t="n">
+        <v>152</v>
+      </c>
+      <c r="B198" s="5" t="inlineStr">
+        <is>
+          <t>Tram acceleration / braking maxima</t>
+        </is>
+      </c>
+      <c r="C198" s="5" t="inlineStr">
+        <is>
+          <t>1.80 / −2.31</t>
+        </is>
+      </c>
+      <c r="D198" s="5" t="inlineStr">
+        <is>
+          <t>m/s²</t>
+        </is>
+      </c>
+      <c r="E198" s="5" t="inlineStr">
+        <is>
+          <t>Same study</t>
+        </is>
+      </c>
+      <c r="F198" s="5" t="inlineStr">
+        <is>
+          <t>Public transport perturbation 2020</t>
+        </is>
+      </c>
+      <c r="G198" s="5" t="inlineStr">
+        <is>
+          <t>(authors not visible in the abstract) (2020). "Perturbation in public transport as a basic concept for perturbation-based balance training for fall prevention". Z. Gerontol. Geriatr..</t>
+        </is>
+      </c>
+      <c r="H198" s="5" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I198" s="6" t="inlineStr">
+        <is>
+          <t>https://link.springer.com/journal/391</t>
+        </is>
+      </c>
+      <c r="J198" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>Perry &amp; Burnfield 2010  —  SLACK Inc.</t>
+        </is>
+      </c>
+      <c r="B199" s="3" t="n"/>
+      <c r="C199" s="3" t="n"/>
+      <c r="D199" s="3" t="n"/>
+      <c r="E199" s="3" t="n"/>
+      <c r="F199" s="3" t="n"/>
+      <c r="G199" s="3" t="n"/>
+      <c r="H199" s="3" t="n"/>
+      <c r="I199" s="3" t="n"/>
+      <c r="J199" s="4" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="5" t="n">
+        <v>153</v>
+      </c>
+      <c r="B200" s="5" t="inlineStr">
+        <is>
+          <t>Gait phases: double support / loading response / toe-off</t>
+        </is>
+      </c>
+      <c r="C200" s="5" t="inlineStr">
+        <is>
+          <t>0–10 % and 50–60 % / 0–10 % / 60 %</t>
+        </is>
+      </c>
+      <c r="D200" s="5" t="inlineStr">
+        <is>
+          <t>% of stride</t>
+        </is>
+      </c>
+      <c r="E200" s="5" t="inlineStr">
+        <is>
+          <t>Normal walking</t>
+        </is>
+      </c>
+      <c r="F200" s="5" t="inlineStr">
+        <is>
+          <t>Perry &amp; Burnfield 2010</t>
+        </is>
+      </c>
+      <c r="G200" s="5" t="inlineStr">
+        <is>
+          <t>J. Perry, J. M. Burnfield (2010). "Gait Analysis: Normal and Pathological Function, 2nd ed.". SLACK Inc..</t>
+        </is>
+      </c>
+      <c r="H200" s="5" t="inlineStr">
+        <is>
+          <t>Textbook</t>
+        </is>
+      </c>
+      <c r="I200" s="6" t="inlineStr">
+        <is>
+          <t>https://www.healio.com/books</t>
+        </is>
+      </c>
+      <c r="J200" s="5" t="inlineStr">
+        <is>
+          <t>Yes (in model, Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t>Krašna et al. 2021  —  Frontiers in Bioengineering and Biotechnology 9:680883</t>
+        </is>
+      </c>
+      <c r="B201" s="3" t="n"/>
+      <c r="C201" s="3" t="n"/>
+      <c r="D201" s="3" t="n"/>
+      <c r="E201" s="3" t="n"/>
+      <c r="F201" s="3" t="n"/>
+      <c r="G201" s="3" t="n"/>
+      <c r="H201" s="3" t="n"/>
+      <c r="I201" s="3" t="n"/>
+      <c r="J201" s="4" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="5" t="n">
+        <v>154</v>
+      </c>
+      <c r="B202" s="5" t="inlineStr">
+        <is>
+          <t>Standing-passenger perturbation pulses tested</t>
+        </is>
+      </c>
+      <c r="C202" s="5" t="inlineStr">
+        <is>
+          <t>1.5 and 3.0 (acc.), 1.0 and 2.5 (braking)</t>
+        </is>
+      </c>
+      <c r="D202" s="5" t="inlineStr">
+        <is>
+          <t>m/s²</t>
+        </is>
+      </c>
+      <c r="E202" s="5" t="inlineStr">
+        <is>
+          <t>Sled tests, 24 volunteers</t>
+        </is>
+      </c>
+      <c r="F202" s="5" t="inlineStr">
+        <is>
+          <t>Krašna et al. 2021</t>
+        </is>
+      </c>
+      <c r="G202" s="5" t="inlineStr">
+        <is>
+          <t>S. Krašna, et al. (2021). "Human Response to Longitudinal Perturbations of Standing Passengers on Public Transport During Regular Operation". Frontiers in Bioengineering and Biotechnology 9:680883.</t>
+        </is>
+      </c>
+      <c r="H202" s="5" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I202" s="6" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3389/fbioe.2021.680883</t>
+        </is>
+      </c>
+      <c r="J202" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
+          <t>Kwok et al. 2015  —  American Journal of Infection Control 43(2):112-114</t>
+        </is>
+      </c>
+      <c r="B203" s="3" t="n"/>
+      <c r="C203" s="3" t="n"/>
+      <c r="D203" s="3" t="n"/>
+      <c r="E203" s="3" t="n"/>
+      <c r="F203" s="3" t="n"/>
+      <c r="G203" s="3" t="n"/>
+      <c r="H203" s="3" t="n"/>
+      <c r="I203" s="3" t="n"/>
+      <c r="J203" s="4" t="n"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="5" t="n">
+        <v>155</v>
+      </c>
+      <c r="B204" s="5" t="inlineStr">
+        <is>
+          <t>Face touching</t>
+        </is>
+      </c>
+      <c r="C204" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="D204" s="5" t="inlineStr">
+        <is>
+          <t>per hour</t>
+        </is>
+      </c>
+      <c r="E204" s="5" t="inlineStr">
+        <is>
+          <t>26 students in a lecture</t>
+        </is>
+      </c>
+      <c r="F204" s="5" t="inlineStr">
+        <is>
+          <t>Kwok et al. 2015</t>
+        </is>
+      </c>
+      <c r="G204" s="5" t="inlineStr">
+        <is>
+          <t>Y. L. A. Kwok, J. Gralton, M.-L. McLaws (2015). "Face touching: a frequent habit that has implications for hand hygiene". American Journal of Infection Control 43(2):112-114.</t>
+        </is>
+      </c>
+      <c r="H204" s="5" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I204" s="6" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.ajic.2014.10.015</t>
+        </is>
+      </c>
+      <c r="J204" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>Mow et al. 2024  —  Proc. ICE Municipal Engineer</t>
+        </is>
+      </c>
+      <c r="B205" s="3" t="n"/>
+      <c r="C205" s="3" t="n"/>
+      <c r="D205" s="3" t="n"/>
+      <c r="E205" s="3" t="n"/>
+      <c r="F205" s="3" t="n"/>
+      <c r="G205" s="3" t="n"/>
+      <c r="H205" s="3" t="n"/>
+      <c r="I205" s="3" t="n"/>
+      <c r="J205" s="4" t="n"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="5" t="n">
+        <v>156</v>
+      </c>
+      <c r="B206" s="5" t="inlineStr">
+        <is>
+          <t>Train-interior touches per passenger movement</t>
+        </is>
+      </c>
+      <c r="C206" s="5" t="inlineStr">
+        <is>
+          <t>0.07 – 0.57</t>
+        </is>
+      </c>
+      <c r="D206" s="5" t="inlineStr">
+        <is>
+          <t>touches</t>
+        </is>
+      </c>
+      <c r="E206" s="5" t="inlineStr">
+        <is>
+          <t>London Underground, 16,891 passengers</t>
+        </is>
+      </c>
+      <c r="F206" s="5" t="inlineStr">
+        <is>
+          <t>Mow et al. 2024</t>
+        </is>
+      </c>
+      <c r="G206" s="5" t="inlineStr">
+        <is>
+          <t>S. Mow, S. Seriani, T. Fujiyama (2024). "Where and how often do people touch train interiors? An investigation during the pandemic". Proc. ICE Municipal Engineer.</t>
+        </is>
+      </c>
+      <c r="H206" s="5" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I206" s="6" t="inlineStr">
+        <is>
+          <t>https://discovery.ucl.ac.uk/id/eprint/10199779/</t>
+        </is>
+      </c>
+      <c r="J206" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>BMRCL EIA  —  BMRCL / JICA</t>
+        </is>
+      </c>
+      <c r="B207" s="3" t="n"/>
+      <c r="C207" s="3" t="n"/>
+      <c r="D207" s="3" t="n"/>
+      <c r="E207" s="3" t="n"/>
+      <c r="F207" s="3" t="n"/>
+      <c r="G207" s="3" t="n"/>
+      <c r="H207" s="3" t="n"/>
+      <c r="I207" s="3" t="n"/>
+      <c r="J207" s="4" t="n"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="5" t="n">
+        <v>157</v>
+      </c>
+      <c r="B208" s="5" t="inlineStr">
+        <is>
+          <t>Bengaluru Metro design loads (standing)</t>
+        </is>
+      </c>
+      <c r="C208" s="5" t="inlineStr">
+        <is>
+          <t>4 / 6 / 8</t>
+        </is>
+      </c>
+      <c r="D208" s="5" t="inlineStr">
+        <is>
+          <t>per m²</t>
+        </is>
+      </c>
+      <c r="E208" s="5" t="inlineStr">
+        <is>
+          <t>Normal / crush / dense crush</t>
+        </is>
+      </c>
+      <c r="F208" s="5" t="inlineStr">
+        <is>
+          <t>BMRCL EIA</t>
+        </is>
+      </c>
+      <c r="G208" s="5" t="inlineStr">
+        <is>
+          <t>Bangalore Metro Rail Corporation Ltd. (n.d.). "Environmental Impact Assessment (design passenger loads)". BMRCL / JICA.</t>
+        </is>
+      </c>
+      <c r="H208" s="5" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="I208" s="6" t="inlineStr">
+        <is>
+          <t>https://www.jica.go.jp/</t>
+        </is>
+      </c>
+      <c r="J208" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t>ISEC WP 437 (2019)  —  ISEC</t>
+        </is>
+      </c>
+      <c r="B209" s="3" t="n"/>
+      <c r="C209" s="3" t="n"/>
+      <c r="D209" s="3" t="n"/>
+      <c r="E209" s="3" t="n"/>
+      <c r="F209" s="3" t="n"/>
+      <c r="G209" s="3" t="n"/>
+      <c r="H209" s="3" t="n"/>
+      <c r="I209" s="3" t="n"/>
+      <c r="J209" s="4" t="n"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="5" t="n">
+        <v>158</v>
+      </c>
+      <c r="B210" s="5" t="inlineStr">
+        <is>
+          <t>One-way commute in Bengaluru</t>
+        </is>
+      </c>
+      <c r="C210" s="5" t="n">
+        <v>42.45</v>
+      </c>
+      <c r="D210" s="5" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="E210" s="5" t="inlineStr">
+        <is>
+          <t>10.84 km average</t>
+        </is>
+      </c>
+      <c r="F210" s="5" t="inlineStr">
+        <is>
+          <t>ISEC WP 437 (2019)</t>
+        </is>
+      </c>
+      <c r="G210" s="5" t="inlineStr">
+        <is>
+          <t>Institute for Social and Economic Change (2019). "Determinants of intra-urban mobility: a study of Bengaluru (Working Paper 437)". ISEC.</t>
+        </is>
+      </c>
+      <c r="H210" s="5" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I210" s="6" t="inlineStr">
+        <is>
+          <t>https://ideas.repec.org/p/sch/wpaper/437.html</t>
+        </is>
+      </c>
+      <c r="J210" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>Espressif ESP-FAQ  —  Espressif documentation</t>
+        </is>
+      </c>
+      <c r="B211" s="3" t="n"/>
+      <c r="C211" s="3" t="n"/>
+      <c r="D211" s="3" t="n"/>
+      <c r="E211" s="3" t="n"/>
+      <c r="F211" s="3" t="n"/>
+      <c r="G211" s="3" t="n"/>
+      <c r="H211" s="3" t="n"/>
+      <c r="I211" s="3" t="n"/>
+      <c r="J211" s="4" t="n"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="5" t="n">
+        <v>159</v>
+      </c>
+      <c r="B212" s="5" t="inlineStr">
+        <is>
+          <t>ESP32 SAR ADC sample-and-hold capacitance</t>
+        </is>
+      </c>
+      <c r="C212" s="5" t="inlineStr">
+        <is>
+          <t>≈ 1</t>
+        </is>
+      </c>
+      <c r="D212" s="5" t="inlineStr">
+        <is>
+          <t>pF</t>
+        </is>
+      </c>
+      <c r="E212" s="5" t="inlineStr"/>
+      <c r="F212" s="5" t="inlineStr">
+        <is>
+          <t>Espressif ESP-FAQ</t>
+        </is>
+      </c>
+      <c r="G212" s="5" t="inlineStr">
+        <is>
+          <t>Espressif Systems (n.d.). "ESP-FAQ: ADC". Espressif documentation.</t>
+        </is>
+      </c>
+      <c r="H212" s="5" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="I212" s="6" t="inlineStr">
+        <is>
+          <t>https://docs.espressif.com/projects/esp-faq/</t>
+        </is>
+      </c>
+      <c r="J212" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>Step-to-Charge 2024  —  arXiv:2408.01927</t>
+        </is>
+      </c>
+      <c r="B213" s="3" t="n"/>
+      <c r="C213" s="3" t="n"/>
+      <c r="D213" s="3" t="n"/>
+      <c r="E213" s="3" t="n"/>
+      <c r="F213" s="3" t="n"/>
+      <c r="G213" s="3" t="n"/>
+      <c r="H213" s="3" t="n"/>
+      <c r="I213" s="3" t="n"/>
+      <c r="J213" s="4" t="n"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="5" t="n">
+        <v>160</v>
+      </c>
+      <c r="B214" s="5" t="inlineStr">
+        <is>
+          <t>Wearable floating ground to earth</t>
+        </is>
+      </c>
+      <c r="C214" s="5" t="inlineStr">
+        <is>
+          <t>≤ 1</t>
+        </is>
+      </c>
+      <c r="D214" s="5" t="inlineStr">
+        <is>
+          <t>pF</t>
+        </is>
+      </c>
+      <c r="E214" s="5" t="inlineStr">
+        <is>
+          <t>Wearable form factors</t>
+        </is>
+      </c>
+      <c r="F214" s="5" t="inlineStr">
+        <is>
+          <t>Step-to-Charge 2024</t>
+        </is>
+      </c>
+      <c r="G214" s="5" t="inlineStr">
+        <is>
+          <t>(Sen group, Purdue) (2024). "Step-to-Charge (EQS body powering)". arXiv:2408.01927.</t>
+        </is>
+      </c>
+      <c r="H214" s="5" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I214" s="6" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2408.01927</t>
+        </is>
+      </c>
+      <c r="J214" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>IEC 61000-4-2  —  International standard</t>
+        </is>
+      </c>
+      <c r="B215" s="3" t="n"/>
+      <c r="C215" s="3" t="n"/>
+      <c r="D215" s="3" t="n"/>
+      <c r="E215" s="3" t="n"/>
+      <c r="F215" s="3" t="n"/>
+      <c r="G215" s="3" t="n"/>
+      <c r="H215" s="3" t="n"/>
+      <c r="I215" s="3" t="n"/>
+      <c r="J215" s="4" t="n"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="5" t="n">
+        <v>161</v>
+      </c>
+      <c r="B216" s="5" t="inlineStr">
+        <is>
+          <t>Human-body model (test standard)</t>
+        </is>
+      </c>
+      <c r="C216" s="5" t="inlineStr">
+        <is>
+          <t>150 pF, 330 Ω</t>
+        </is>
+      </c>
+      <c r="D216" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E216" s="5" t="inlineStr">
+        <is>
+          <t>Discharge time constant ≈ 50 ns; rise time 0.8 ns ±25 %</t>
+        </is>
+      </c>
+      <c r="F216" s="5" t="inlineStr">
+        <is>
+          <t>IEC 61000-4-2</t>
+        </is>
+      </c>
+      <c r="G216" s="5" t="inlineStr">
+        <is>
+          <t>IEC (2008). "IEC 61000-4-2: Electrostatic discharge immunity test". International standard.</t>
+        </is>
+      </c>
+      <c r="H216" s="5" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I216" s="6" t="inlineStr">
+        <is>
+          <t>https://webstore.iec.ch/publication/4189</t>
+        </is>
+      </c>
+      <c r="J216" s="5" t="inlineStr">
+        <is>
+          <t>Yes (in model, Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>Ramallah ELF survey  —  Journal article</t>
+        </is>
+      </c>
+      <c r="B217" s="3" t="n"/>
+      <c r="C217" s="3" t="n"/>
+      <c r="D217" s="3" t="n"/>
+      <c r="E217" s="3" t="n"/>
+      <c r="F217" s="3" t="n"/>
+      <c r="G217" s="3" t="n"/>
+      <c r="H217" s="3" t="n"/>
+      <c r="I217" s="3" t="n"/>
+      <c r="J217" s="4" t="n"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="5" t="n">
+        <v>162</v>
+      </c>
+      <c r="B218" s="5" t="inlineStr">
+        <is>
+          <t>Indoor 50 Hz electric field in homes, geometric mean</t>
+        </is>
+      </c>
+      <c r="C218" s="5" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="D218" s="5" t="inlineStr">
+        <is>
+          <t>V/m</t>
+        </is>
+      </c>
+      <c r="E218" s="5" t="inlineStr">
+        <is>
+          <t>32 homes, log-normal</t>
+        </is>
+      </c>
+      <c r="F218" s="5" t="inlineStr">
+        <is>
+          <t>Ramallah ELF survey</t>
+        </is>
+      </c>
+      <c r="G218" s="5" t="inlineStr">
+        <is>
+          <t>(Al-Quds / An-Najah University) (n.d.). "Residential exposure to ELF electric and magnetic fields in the city of Ramallah-Palestine". Journal article.</t>
+        </is>
+      </c>
+      <c r="H218" s="5" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I218" s="6" t="inlineStr">
+        <is>
+          <t>https://dspace.alquds.edu/items/bc4377ca-bfb7-4375-ab1a-435c8e020c57/full</t>
+        </is>
+      </c>
+      <c r="J218" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>Aziz et al. 2017  —  PLoS ONE 12(7):e0180318</t>
+        </is>
+      </c>
+      <c r="B219" s="3" t="n"/>
+      <c r="C219" s="3" t="n"/>
+      <c r="D219" s="3" t="n"/>
+      <c r="E219" s="3" t="n"/>
+      <c r="F219" s="3" t="n"/>
+      <c r="G219" s="3" t="n"/>
+      <c r="H219" s="3" t="n"/>
+      <c r="I219" s="3" t="n"/>
+      <c r="J219" s="4" t="n"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="5" t="n">
+        <v>163</v>
+      </c>
+      <c r="B220" s="5" t="inlineStr">
+        <is>
+          <t>Fall-detector false alarms, real-world</t>
+        </is>
+      </c>
+      <c r="C220" s="5" t="inlineStr">
+        <is>
+          <t>0 – 0.3</t>
+        </is>
+      </c>
+      <c r="D220" s="5" t="inlineStr">
+        <is>
+          <t>per hour</t>
+        </is>
+      </c>
+      <c r="E220" s="5" t="inlineStr">
+        <is>
+          <t>≈ 400 h, waist/sternum</t>
+        </is>
+      </c>
+      <c r="F220" s="5" t="inlineStr">
+        <is>
+          <t>Aziz et al. 2017</t>
+        </is>
+      </c>
+      <c r="G220" s="5" t="inlineStr">
+        <is>
+          <t>O. Aziz, et al. (2017). "Validation of accuracy of SVM-based fall detection system using real-world fall and non-fall datasets". PLoS ONE 12(7):e0180318.</t>
+        </is>
+      </c>
+      <c r="H220" s="5" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I220" s="6" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1371/journal.pone.0180318</t>
+        </is>
+      </c>
+      <c r="J220" s="5" t="inlineStr">
+        <is>
+          <t>Accuracy benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="inlineStr">
+        <is>
+          <t>Indraganti et al. 2014  —  Windsor Conference</t>
+        </is>
+      </c>
+      <c r="B221" s="3" t="n"/>
+      <c r="C221" s="3" t="n"/>
+      <c r="D221" s="3" t="n"/>
+      <c r="E221" s="3" t="n"/>
+      <c r="F221" s="3" t="n"/>
+      <c r="G221" s="3" t="n"/>
+      <c r="H221" s="3" t="n"/>
+      <c r="I221" s="3" t="n"/>
+      <c r="J221" s="4" t="n"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="5" t="n">
+        <v>164</v>
+      </c>
+      <c r="B222" s="5" t="inlineStr">
+        <is>
+          <t>Thermal insulation of a sari, by drape</t>
+        </is>
+      </c>
+      <c r="C222" s="5" t="inlineStr">
+        <is>
+          <t>0.62 – 0.94</t>
+        </is>
+      </c>
+      <c r="D222" s="5" t="inlineStr">
+        <is>
+          <t>clo</t>
+        </is>
+      </c>
+      <c r="E222" s="5" t="inlineStr">
+        <is>
+          <t>Manikin, ISO 9920</t>
+        </is>
+      </c>
+      <c r="F222" s="5" t="inlineStr">
+        <is>
+          <t>Indraganti et al. 2014</t>
+        </is>
+      </c>
+      <c r="G222" s="5" t="inlineStr">
+        <is>
+          <t>M. Indraganti, et al. (2014). "Thermal insulation of Indian clothing ensembles (sari, salwar-kurti)". Windsor Conference.</t>
+        </is>
+      </c>
+      <c r="H222" s="5" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I222" s="6" t="inlineStr">
+        <is>
+          <t>https://architexturez.net/node/175314</t>
+        </is>
+      </c>
+      <c r="J222" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t>Majumdar et al. (Hyderabad)  —  Transportation Research Record</t>
+        </is>
+      </c>
+      <c r="B223" s="3" t="n"/>
+      <c r="C223" s="3" t="n"/>
+      <c r="D223" s="3" t="n"/>
+      <c r="E223" s="3" t="n"/>
+      <c r="F223" s="3" t="n"/>
+      <c r="G223" s="3" t="n"/>
+      <c r="H223" s="3" t="n"/>
+      <c r="I223" s="3" t="n"/>
+      <c r="J223" s="4" t="n"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="5" t="n">
+        <v>165</v>
+      </c>
+      <c r="B224" s="5" t="inlineStr">
+        <is>
+          <t>Physical harassment in public transport: touching / groping</t>
+        </is>
+      </c>
+      <c r="C224" s="5" t="inlineStr">
+        <is>
+          <t>58.8 / 53.2</t>
+        </is>
+      </c>
+      <c r="D224" s="5" t="inlineStr">
+        <is>
+          <t>% of victims</t>
+        </is>
+      </c>
+      <c r="E224" s="5" t="inlineStr">
+        <is>
+          <t>Hyderabad, 583 respondents; Secondary</t>
+        </is>
+      </c>
+      <c r="F224" s="5" t="inlineStr">
+        <is>
+          <t>Majumdar et al. (Hyderabad)</t>
+        </is>
+      </c>
+      <c r="G224" s="5" t="inlineStr">
+        <is>
+          <t>B. B. Majumdar, et al. (BITS Pilani Hyderabad) (n.d.). "Harassment of women in public transport, Hyderabad". Transportation Research Record.</t>
+        </is>
+      </c>
+      <c r="H224" s="5" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="I224" s="6" t="inlineStr">
+        <is>
+          <t>https://journals.sagepub.com/home/trr</t>
+        </is>
+      </c>
+      <c r="J224" s="5" t="inlineStr">
+        <is>
+          <t>Background only</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J161"/>
-  <mergeCells count="31">
+  <autoFilter ref="A1:J224"/>
+  <mergeCells count="58">
+    <mergeCell ref="A203:J203"/>
     <mergeCell ref="A160:J160"/>
     <mergeCell ref="A23:J23"/>
+    <mergeCell ref="A194:J194"/>
     <mergeCell ref="A141:J141"/>
+    <mergeCell ref="A219:J219"/>
     <mergeCell ref="A150:J150"/>
+    <mergeCell ref="A188:J188"/>
+    <mergeCell ref="A213:J213"/>
+    <mergeCell ref="A215:J215"/>
     <mergeCell ref="A109:J109"/>
+    <mergeCell ref="A180:J180"/>
     <mergeCell ref="A156:J156"/>
     <mergeCell ref="A125:J125"/>
+    <mergeCell ref="A171:J171"/>
+    <mergeCell ref="A209:J209"/>
     <mergeCell ref="A134:J134"/>
+    <mergeCell ref="A199:J199"/>
     <mergeCell ref="A152:J152"/>
     <mergeCell ref="A115:J115"/>
     <mergeCell ref="A31:J31"/>
+    <mergeCell ref="A167:J167"/>
+    <mergeCell ref="A173:J173"/>
+    <mergeCell ref="A211:J211"/>
     <mergeCell ref="A148:J148"/>
+    <mergeCell ref="A186:J186"/>
     <mergeCell ref="A73:J73"/>
+    <mergeCell ref="A201:J201"/>
+    <mergeCell ref="A182:J182"/>
     <mergeCell ref="A98:J98"/>
     <mergeCell ref="A60:J60"/>
+    <mergeCell ref="A169:J169"/>
     <mergeCell ref="A49:J49"/>
     <mergeCell ref="A138:J138"/>
+    <mergeCell ref="A207:J207"/>
     <mergeCell ref="A103:J103"/>
     <mergeCell ref="A132:J132"/>
     <mergeCell ref="A79:J79"/>
     <mergeCell ref="A119:J119"/>
+    <mergeCell ref="A162:J162"/>
+    <mergeCell ref="A196:J196"/>
+    <mergeCell ref="A205:J205"/>
+    <mergeCell ref="A221:J221"/>
+    <mergeCell ref="A177:J177"/>
     <mergeCell ref="A90:J90"/>
     <mergeCell ref="A128:J128"/>
     <mergeCell ref="A66:J66"/>
+    <mergeCell ref="A217:J217"/>
     <mergeCell ref="A37:J37"/>
     <mergeCell ref="A145:J145"/>
     <mergeCell ref="A158:J158"/>
     <mergeCell ref="A136:J136"/>
     <mergeCell ref="A154:J154"/>
+    <mergeCell ref="A192:J192"/>
+    <mergeCell ref="A223:J223"/>
     <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A175:J175"/>
     <mergeCell ref="A76:J76"/>
   </mergeCells>
   <hyperlinks>
@@ -7500,6 +9727,42 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I157" r:id="rId127"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I159" r:id="rId128"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I161" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I163" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I164" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I165" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I166" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I168" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I170" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I172" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I174" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I176" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I178" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I179" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I181" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I183" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I184" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I185" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I187" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I189" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I190" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I191" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I193" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I195" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I197" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I198" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I200" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I202" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I204" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I206" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I208" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I210" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I212" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I214" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I216" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I218" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I220" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I222" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I224" r:id="rId165"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7511,7 +9774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -8097,6 +10360,492 @@
         </is>
       </c>
       <c r="D32" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>A. Talebzadeh, M. Moradian, Y. Han, D. E. Swenson, D. Pommerenke (2016). "Effect of Human Activities and Environmental Conditions on Electrostatic Charging". IEEE Trans. Electromagnetic Compatibility 58(4).</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/TEMC.2016.2575842</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>M. Kangas, R. Korpelainen, I. Vikman, L. Nyberg, T. Jämsä (2015). "Sensitivity and false alarm rate of a fall sensor in long-term fall detection in the elderly". Gerontology 61(1):61-68.</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1159/000362720</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>F. Tchuente, N. Baddour, E. D. Lemaire (2020). "Classification of Aggressive Movements Using Smartwatches". Sensors 20(21):6377.</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/s20216377</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>Texas Instruments (2015). "OPA350, OPA2350, OPA4350 high-speed single-supply rail-to-rail operational amplifiers (SBOS099D)". Datasheet.</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>https://www.ti.com/lit/ds/symlink/opa350.pdf</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>ECN / passive-components.eu (using TI figures) (n.d.). "A Plague of Parasites (PCB trace capacitance)". Trade article.</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>https://passive-components.eu/</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>Specialty Coating Systems (n.d.). "Parylene Dielectric Properties". Manufacturer technical data.</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>https://scscoatings.com/</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>A. Visuri, Z. Sarsenbayeva, N. van Berkel, J. Goncalves, R. Rawassizadeh, V. Kostakos, D. Ferreira (2017). "Quantifying Sources and Types of Smartwatch Usage Sessions". Proc. ACM CHI 2017, pp. 3569-3581.</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1145/3025453.3025817</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>S. Andrews, D. A. Ellis, H. Shaw, L. Piwek (2015). "Beyond Self-Report: Tools to Compare Estimated and Real-World Smartphone Use". PLoS ONE 10(10):e0139004.</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1371/journal.pone.0139004</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>T. Ficker (2005). "Charging by walking". J. Phys. D: Appl. Phys. 38(5):410-417.</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>https://incompliancemag.com/charging-by-walking/</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>C. Tudor-Locke, H. Han, E. J. Aguiar, et al. (2012). "Using cadence to study free-living ambulatory activity". Sports Medicine 42(5):381-398.</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>https://strathprints.strath.ac.uk/42646/</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>D. Neacsu, A. Salceanu, E. Lunca, V. David (2007). "Indirect Measurements on the Capacity in the Electrostatic HB Model". IMEKO TC4 Symposium, Iasi.</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>https://imeko.org/proceedings/indirect-measurements-on-the-capacity-in-the-electrostatic-hb-model</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>N. P. Dawkins, T. Yates, et al. (2022). "Normative wrist-worn accelerometer values for self-paced walking and running: a walk in the park". J. Sports Sciences.</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1080/02640414.2021.1976491</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>(authors as listed on arXiv) (2022). "A 'one-size-fits-most' walking recognition method for smartphones, smartwatches, and wearable accelerometers". arXiv:2207.07443.</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2207.07443</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>(authors not visible in the abstract) (2020). "Perturbation in public transport as a basic concept for perturbation-based balance training for fall prevention". Z. Gerontol. Geriatr..</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>https://link.springer.com/journal/391</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>J. Perry, J. M. Burnfield (2010). "Gait Analysis: Normal and Pathological Function, 2nd ed.". SLACK Inc..</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>https://www.healio.com/books</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>S. Krašna, et al. (2021). "Human Response to Longitudinal Perturbations of Standing Passengers on Public Transport During Regular Operation". Frontiers in Bioengineering and Biotechnology 9:680883.</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3389/fbioe.2021.680883</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>Y. L. A. Kwok, J. Gralton, M.-L. McLaws (2015). "Face touching: a frequent habit that has implications for hand hygiene". American Journal of Infection Control 43(2):112-114.</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.ajic.2014.10.015</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>S. Mow, S. Seriani, T. Fujiyama (2024). "Where and how often do people touch train interiors? An investigation during the pandemic". Proc. ICE Municipal Engineer.</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>https://discovery.ucl.ac.uk/id/eprint/10199779/</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>Bangalore Metro Rail Corporation Ltd. (n.d.). "Environmental Impact Assessment (design passenger loads)". BMRCL / JICA.</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>https://www.jica.go.jp/</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>Institute for Social and Economic Change (2019). "Determinants of intra-urban mobility: a study of Bengaluru (Working Paper 437)". ISEC.</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>https://ideas.repec.org/p/sch/wpaper/437.html</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>Espressif Systems (n.d.). "ESP-FAQ: ADC". Espressif documentation.</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>https://docs.espressif.com/projects/esp-faq/</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>(Sen group, Purdue) (2024). "Step-to-Charge (EQS body powering)". arXiv:2408.01927.</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2408.01927</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>IEC (2008). "IEC 61000-4-2: Electrostatic discharge immunity test". International standard.</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="inlineStr">
+        <is>
+          <t>https://webstore.iec.ch/publication/4189</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>(Al-Quds / An-Najah University) (n.d.). "Residential exposure to ELF electric and magnetic fields in the city of Ramallah-Palestine". Journal article.</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>https://dspace.alquds.edu/items/bc4377ca-bfb7-4375-ab1a-435c8e020c57/full</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>O. Aziz, et al. (2017). "Validation of accuracy of SVM-based fall detection system using real-world fall and non-fall datasets". PLoS ONE 12(7):e0180318.</t>
+        </is>
+      </c>
+      <c r="C57" s="9" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1371/journal.pone.0180318</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>M. Indraganti, et al. (2014). "Thermal insulation of Indian clothing ensembles (sari, salwar-kurti)". Windsor Conference.</t>
+        </is>
+      </c>
+      <c r="C58" s="9" t="inlineStr">
+        <is>
+          <t>https://architexturez.net/node/175314</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="8" t="inlineStr">
+        <is>
+          <t>B. B. Majumdar, et al. (BITS Pilani Hyderabad) (n.d.). "Harassment of women in public transport, Hyderabad". Transportation Research Record.</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
+        <is>
+          <t>https://journals.sagepub.com/home/trr</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8133,6 +10882,33 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId58"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Explorer: numbered References section (IEEE style) with in-text citations
The References list at the bottom of the page shows on every tab: [n] is source Sn of
docs/parameter_sources.md and the workbook, formatted as authors, "title," venue, year, DOI or
link. Statements on the page cite their sources as [n] links. Adds FastCap (Nabors & White
1991) and the ngspice manual as sources S59, S60. Replaces the searchable References tab.
</commit_message>
<xml_diff>
--- a/docs/SparshaGuard_paper_values.xlsx
+++ b/docs/SparshaGuard_paper_values.xlsx
@@ -9774,7 +9774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -10847,6 +10847,42 @@
       </c>
       <c r="D59" s="8" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>K. Nabors, J. White (1991). "FastCap: A Multipole Accelerated 3-D Capacitance Extraction Program". IEEE Trans. Computer-Aided Design 10(11):1447-1459.</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/43.97624</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="8" t="inlineStr">
+        <is>
+          <t>H. Vogt, G. Atkinson, P. Nenzi (n.d.). "Ngspice User's Manual". ngspice project.</t>
+        </is>
+      </c>
+      <c r="C61" s="9" t="inlineStr">
+        <is>
+          <t>https://ngspice.sourceforge.io/docs.html</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -10909,6 +10945,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId60"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>